<commit_message>
Removed completed jobs 29/7/26
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CED83A92-01AD-456D-B8A3-C2FA243C4A99}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DFA43EA-996D-40BE-BE3C-35083BDCFAA8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="329">
   <si>
     <t>Job</t>
   </si>
@@ -59,9 +59,6 @@
     <t>1084466 - 00057025 - DG Label</t>
   </si>
   <si>
-    <t>1084465 - 00053318 - DG Label</t>
-  </si>
-  <si>
     <t>1084464 - 00050442 - DG Label</t>
   </si>
   <si>
@@ -86,33 +83,15 @@
     <t>9 Kaka Road, Taihape</t>
   </si>
   <si>
-    <t>1084304 - 00053706 - DG Label</t>
-  </si>
-  <si>
     <t>1084171 - 00014163 - DG Label</t>
   </si>
   <si>
-    <t>1084166 - 00020534 - DG Label</t>
-  </si>
-  <si>
-    <t>1084164 - 00045748 - DG Label</t>
-  </si>
-  <si>
-    <t>1084162 - 00035457 - DG Label</t>
-  </si>
-  <si>
-    <t>1933 SH 3, Turakina</t>
-  </si>
-  <si>
     <t>1084156 - 00027186 - DG Label</t>
   </si>
   <si>
     <t>The Lido</t>
   </si>
   <si>
-    <t>1084084 - 00057184 - DG Label</t>
-  </si>
-  <si>
     <t>1084083 - 00057507 - DG Label</t>
   </si>
   <si>
@@ -125,12 +104,6 @@
     <t>1084079 - 00059083 - DG Label</t>
   </si>
   <si>
-    <t>1084060 - 00023511 - DG Label</t>
-  </si>
-  <si>
-    <t>289 Kairanga Bunnythorpe Road</t>
-  </si>
-  <si>
     <t>1084059 - 00051796 - DG Label</t>
   </si>
   <si>
@@ -164,24 +137,12 @@
     <t>49 Weld Street, Martinborough</t>
   </si>
   <si>
-    <t>1083911 - 00055085 - DG Label</t>
-  </si>
-  <si>
-    <t>171 Great North Road, Otamatea</t>
-  </si>
-  <si>
     <t>1083909 - 00051891 - DG Label</t>
   </si>
   <si>
     <t>16 Mersey Street, Rongotea</t>
   </si>
   <si>
-    <t>1083907 - 00044159 - DG Label</t>
-  </si>
-  <si>
-    <t>11 Springwater Drive, Feilding</t>
-  </si>
-  <si>
     <t>1083906 - 00047054 - DG Label</t>
   </si>
   <si>
@@ -212,12 +173,6 @@
     <t>290D Dakins Road, Carterton</t>
   </si>
   <si>
-    <t>1083716 - 00054934 - DG Label</t>
-  </si>
-  <si>
-    <t>57 Somerset Road, Springvale</t>
-  </si>
-  <si>
     <t>1083715 - 00056130 - DG Label</t>
   </si>
   <si>
@@ -272,24 +227,12 @@
     <t>10 Alton Grove, Masterton</t>
   </si>
   <si>
-    <t>1083701 - 00027885 - DG Label</t>
-  </si>
-  <si>
-    <t>110 Port Street East, Feilding</t>
-  </si>
-  <si>
     <t>1083699 - 00059938 - DG Label</t>
   </si>
   <si>
     <t>1009 Taonui Road, Colyton</t>
   </si>
   <si>
-    <t>1083698 - 00051118 - DG Label</t>
-  </si>
-  <si>
-    <t>21 Waharua Place, Tawhero</t>
-  </si>
-  <si>
     <t>1083697 - 00050711 - DG Label</t>
   </si>
   <si>
@@ -302,12 +245,6 @@
     <t>48 Raetihi Ohakune Road, Raetihi</t>
   </si>
   <si>
-    <t>1083656 - 00055415 - DG Label</t>
-  </si>
-  <si>
-    <t>46 Tongariro Street, Castlecliff</t>
-  </si>
-  <si>
     <t>1083539 - 00047551 - DG Label</t>
   </si>
   <si>
@@ -476,12 +413,6 @@
     <t>16 Parkers Road, Carterton</t>
   </si>
   <si>
-    <t>1083187 - 00047452 - DG Label</t>
-  </si>
-  <si>
-    <t>5 Ferndale Place, Feilding</t>
-  </si>
-  <si>
     <t>1083186 - 00051708 - DG Label</t>
   </si>
   <si>
@@ -521,12 +452,6 @@
     <t>20 Langley Avenue, Milson</t>
   </si>
   <si>
-    <t>1083028 - 00033796 - DG Label</t>
-  </si>
-  <si>
-    <t>243 Napier Road, Kelvin Grove</t>
-  </si>
-  <si>
     <t>1083023 - 00022620 - DG Label</t>
   </si>
   <si>
@@ -557,18 +482,6 @@
     <t>429A Black Rock Road, Masterton</t>
   </si>
   <si>
-    <t>1082796 - 00041294 - DG Label</t>
-  </si>
-  <si>
-    <t>27A Parrs Road, Bunnythorpe, 4470</t>
-  </si>
-  <si>
-    <t>1082794 - 00025227 - DG Label</t>
-  </si>
-  <si>
-    <t>1C WYNDHAM STREET, ASHHURST, 4810</t>
-  </si>
-  <si>
     <t>1082793 - 00047634 - DG Label</t>
   </si>
   <si>
@@ -686,21 +599,6 @@
     <t>1082300 - 00046363 - DG Label</t>
   </si>
   <si>
-    <t>1082226 - 00041473 - DG Label</t>
-  </si>
-  <si>
-    <t>1082225 - 00051233 - DG Label</t>
-  </si>
-  <si>
-    <t>7 OAK CRES, ASHHURST</t>
-  </si>
-  <si>
-    <t>1082224 - 00052577 - DG Label</t>
-  </si>
-  <si>
-    <t>1055 VALLEY RD, ASHHURST</t>
-  </si>
-  <si>
     <t>1082166 - 00052136 - DG Label</t>
   </si>
   <si>
@@ -797,18 +695,6 @@
     <t>34 Jellicoe Street, Martinborough</t>
   </si>
   <si>
-    <t>1082676 - 00055845 - DG Label - 0000022362CPC8E</t>
-  </si>
-  <si>
-    <t>346 Botanical Road, Palmerston North</t>
-  </si>
-  <si>
-    <t>1082649 - 00040553 - DG Label -0900085009PC066</t>
-  </si>
-  <si>
-    <t>14 PARNELL HEIGHTS DRIVE , KELVIN GROVE, PALMERSTON NORTH, 4414</t>
-  </si>
-  <si>
     <t>1082613 - 00037301  - DG Label - 0068841000WR999</t>
   </si>
   <si>
@@ -887,12 +773,6 @@
     <t>2 VISCOUNT PLACE, WEST END, PALMERSTON NORTH, 4412</t>
   </si>
   <si>
-    <t>1082566 - 00030742 - DG Label - 0000053096CP589</t>
-  </si>
-  <si>
-    <t>9 PUKETIRO DRIVE, FEILDING, 4702</t>
-  </si>
-  <si>
     <t>1082562 - 00052452 - DG Label - 0000080600CP356</t>
   </si>
   <si>
@@ -935,12 +815,6 @@
     <t>15 RON PLACE, FITZHERBERT, PALMERSTON NORTH, 4410</t>
   </si>
   <si>
-    <t>1082499 - 00052869 - DG Label - 0900090812PCBD3</t>
-  </si>
-  <si>
-    <t>4 STONEBRIDGE HEIGHTS, FEILDING, 4702</t>
-  </si>
-  <si>
     <t>1082492 - 00055639 - DG Label - 0000037890CP0D3</t>
   </si>
   <si>
@@ -968,36 +842,12 @@
     <t>1082477 - 00052899 - DG Label- 1000594314PC4FC</t>
   </si>
   <si>
-    <t>1082475 - 00050997 - DG Label - 0900090099PC040</t>
-  </si>
-  <si>
-    <t>45A SHERWILL STREET EAST, FEILDING, 4702</t>
-  </si>
-  <si>
-    <t>1082462 - 00057612 - DG Label - 1000564472PC01D</t>
-  </si>
-  <si>
-    <t>17 Wescombe Grove, Feilding, 4702</t>
-  </si>
-  <si>
-    <t>1082460 - 00055909 - DG Label - 0000042708CPFB6</t>
-  </si>
-  <si>
-    <t>27 RAILWAY ROAD, PALMERSTON NORTH</t>
-  </si>
-  <si>
     <t>1082458 - 00054943 - DG Label - 1000624687PC063</t>
   </si>
   <si>
     <t>8 Sardinia Grove, Fitzherbert, Palmerston North</t>
   </si>
   <si>
-    <t>1082457 - 00047081 - DG Label - 0000022942CPBD1</t>
-  </si>
-  <si>
-    <t>15 CARDIFF STREET, AWAPUNI, PALMERSTON NORTH, 4412</t>
-  </si>
-  <si>
     <t>1082455 - 00044025 - DG Label - 1000621883PC042</t>
   </si>
   <si>
@@ -1034,9 +884,6 @@
     <t>231 Valley Views, Palmerston North</t>
   </si>
   <si>
-    <t>326 Creek Road, Whanganui</t>
-  </si>
-  <si>
     <t>99A Lees Pakaraka Road, Masterton</t>
   </si>
   <si>
@@ -1049,18 +896,6 @@
     <t>89 Dublin Street, Martinborough</t>
   </si>
   <si>
-    <t>15 Wapiti Avenue, Feilding</t>
-  </si>
-  <si>
-    <t>10 Tangaroa View, Whanganui</t>
-  </si>
-  <si>
-    <t>21 Waipounamu Street, Whanganui</t>
-  </si>
-  <si>
-    <t>49 Hereford Street, Whanganui</t>
-  </si>
-  <si>
     <t>1853 Rongotea Road, Rongotea</t>
   </si>
   <si>
@@ -1076,9 +911,6 @@
     <t>46A Main Street, Greytown</t>
   </si>
   <si>
-    <t>44 LINCOLN STREET, Ashhurst</t>
-  </si>
-  <si>
     <t>95 Pyke Road, Rangitou</t>
   </si>
   <si>
@@ -1109,18 +941,6 @@
     <t>26 MAKOPUA ROAD, TAOROA JUNCTION</t>
   </si>
   <si>
-    <t>1084695 - 00062451 - DG Label</t>
-  </si>
-  <si>
-    <t>10 Webster Place, Otamatea</t>
-  </si>
-  <si>
-    <t>677 Rapanui Road, Wanganui</t>
-  </si>
-  <si>
-    <t>1084696 - 00059596 - DG Label</t>
-  </si>
-  <si>
     <t>45D Brandon Street, Featherston</t>
   </si>
   <si>
@@ -1151,12 +971,6 @@
     <t>1084703 - 00056419 - DG Label</t>
   </si>
   <si>
-    <t>163 Nannestads Line, Feilding</t>
-  </si>
-  <si>
-    <t>1084704 - 00063979 - DG Label</t>
-  </si>
-  <si>
     <t>37 Pukenaua Road, Taihape</t>
   </si>
   <si>
@@ -1172,12 +986,6 @@
     <t>1084709 - 00022620 - DG Label</t>
   </si>
   <si>
-    <t>Aerowork Airport Road, Whanganui</t>
-  </si>
-  <si>
-    <t>1084710 - 233751 - DG Label</t>
-  </si>
-  <si>
     <t>37 Fry Road, Halcombe</t>
   </si>
   <si>
@@ -1212,12 +1020,6 @@
   </si>
   <si>
     <t>1084779 - 00048369 - DG Label</t>
-  </si>
-  <si>
-    <t>75 Somerset Road, Springvale</t>
-  </si>
-  <si>
-    <t>1084780 - 00050330 - DG Label</t>
   </si>
   <si>
     <t>5 Pukeko Place, Riversdale Beach</t>
@@ -1604,7 +1406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C197"/>
+  <dimension ref="A1:C164"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -1620,2163 +1422,1800 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>329</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="B2" t="s">
-        <v>253</v>
+        <v>219</v>
       </c>
       <c r="C2" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>254</v>
+        <v>220</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>221</v>
       </c>
       <c r="C3" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>256</v>
+        <v>222</v>
       </c>
       <c r="B4" t="s">
-        <v>257</v>
+        <v>223</v>
       </c>
       <c r="C4" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>258</v>
+        <v>224</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>225</v>
       </c>
       <c r="C5" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>260</v>
+        <v>226</v>
       </c>
       <c r="B6" t="s">
-        <v>261</v>
+        <v>227</v>
       </c>
       <c r="C6" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>262</v>
+        <v>228</v>
       </c>
       <c r="B7" t="s">
-        <v>263</v>
+        <v>229</v>
       </c>
       <c r="C7" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>264</v>
+        <v>230</v>
       </c>
       <c r="B8" t="s">
-        <v>265</v>
+        <v>231</v>
       </c>
       <c r="C8" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>266</v>
+        <v>232</v>
       </c>
       <c r="B9" t="s">
-        <v>267</v>
+        <v>233</v>
       </c>
       <c r="C9" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>268</v>
+        <v>234</v>
       </c>
       <c r="B10" t="s">
-        <v>269</v>
+        <v>235</v>
       </c>
       <c r="C10" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>270</v>
+        <v>236</v>
       </c>
       <c r="B11" t="s">
-        <v>271</v>
+        <v>237</v>
       </c>
       <c r="C11" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>272</v>
+        <v>238</v>
       </c>
       <c r="B12" t="s">
-        <v>273</v>
+        <v>239</v>
       </c>
       <c r="C12" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>274</v>
+        <v>240</v>
       </c>
       <c r="B13" t="s">
-        <v>275</v>
+        <v>241</v>
       </c>
       <c r="C13" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>276</v>
+        <v>242</v>
       </c>
       <c r="B14" t="s">
-        <v>277</v>
+        <v>243</v>
       </c>
       <c r="C14" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>278</v>
+        <v>244</v>
       </c>
       <c r="B15" t="s">
-        <v>279</v>
+        <v>245</v>
       </c>
       <c r="C15" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>280</v>
+        <v>246</v>
       </c>
       <c r="B16" t="s">
-        <v>281</v>
+        <v>247</v>
       </c>
       <c r="C16" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>282</v>
+        <v>248</v>
       </c>
       <c r="B17" t="s">
-        <v>283</v>
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>284</v>
+        <v>250</v>
       </c>
       <c r="B18" t="s">
-        <v>285</v>
+        <v>251</v>
       </c>
       <c r="C18" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>286</v>
+        <v>252</v>
       </c>
       <c r="B19" t="s">
-        <v>287</v>
+        <v>253</v>
       </c>
       <c r="C19" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>288</v>
+        <v>254</v>
       </c>
       <c r="B20" t="s">
-        <v>289</v>
+        <v>255</v>
       </c>
       <c r="C20" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>290</v>
+        <v>256</v>
       </c>
       <c r="B21" t="s">
-        <v>291</v>
+        <v>257</v>
       </c>
       <c r="C21" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>292</v>
+        <v>258</v>
       </c>
       <c r="B22" t="s">
-        <v>293</v>
+        <v>259</v>
       </c>
       <c r="C22" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>294</v>
+        <v>260</v>
       </c>
       <c r="B23" t="s">
-        <v>295</v>
+        <v>261</v>
       </c>
       <c r="C23" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>296</v>
+        <v>262</v>
       </c>
       <c r="B24" t="s">
-        <v>297</v>
+        <v>263</v>
       </c>
       <c r="C24" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>298</v>
+        <v>264</v>
       </c>
       <c r="B25" t="s">
-        <v>299</v>
+        <v>265</v>
       </c>
       <c r="C25" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>300</v>
+        <v>266</v>
       </c>
       <c r="B26" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C26" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>302</v>
+        <v>267</v>
       </c>
       <c r="B27" t="s">
-        <v>303</v>
+        <v>268</v>
       </c>
       <c r="C27" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>304</v>
+        <v>269</v>
       </c>
       <c r="B28" t="s">
-        <v>305</v>
+        <v>270</v>
       </c>
       <c r="C28" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>306</v>
+        <v>271</v>
       </c>
       <c r="B29" t="s">
-        <v>307</v>
+        <v>272</v>
       </c>
       <c r="C29" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>308</v>
+        <v>273</v>
       </c>
       <c r="B30" t="s">
-        <v>355</v>
+        <v>274</v>
       </c>
       <c r="C30" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>309</v>
+        <v>275</v>
       </c>
       <c r="B31" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="C31" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>311</v>
+        <v>149</v>
       </c>
       <c r="B32" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>313</v>
+        <v>150</v>
       </c>
       <c r="B33" t="s">
-        <v>314</v>
+        <v>151</v>
       </c>
       <c r="C33" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>315</v>
+        <v>152</v>
       </c>
       <c r="B34" t="s">
-        <v>316</v>
+        <v>153</v>
       </c>
       <c r="C34" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>317</v>
+        <v>154</v>
       </c>
       <c r="B35" t="s">
-        <v>318</v>
+        <v>155</v>
       </c>
       <c r="C35" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>319</v>
+        <v>156</v>
       </c>
       <c r="B36" t="s">
-        <v>320</v>
+        <v>157</v>
       </c>
       <c r="C36" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>321</v>
+        <v>158</v>
       </c>
       <c r="B37" t="s">
-        <v>322</v>
+        <v>159</v>
       </c>
       <c r="C37" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>323</v>
+        <v>160</v>
       </c>
       <c r="B38" t="s">
-        <v>324</v>
+        <v>161</v>
       </c>
       <c r="C38" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>325</v>
+        <v>162</v>
       </c>
       <c r="B39" t="s">
-        <v>354</v>
+        <v>163</v>
       </c>
       <c r="C39" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="B40" t="s">
-        <v>353</v>
+        <v>165</v>
       </c>
       <c r="C40" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="B41" t="s">
-        <v>180</v>
+        <v>167</v>
       </c>
       <c r="C41" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>181</v>
+        <v>168</v>
       </c>
       <c r="B42" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C42" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="B43" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C43" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="C44" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="B45" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="C45" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="B46" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="C46" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="B47" t="s">
-        <v>192</v>
+        <v>296</v>
       </c>
       <c r="C47" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="B48" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="C48" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="B49" t="s">
-        <v>196</v>
+        <v>182</v>
       </c>
       <c r="C49" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="B50" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="C50" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="B51" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="C51" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="B52" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C52" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="B53" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C53" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="B54" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C54" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="B55" t="s">
-        <v>352</v>
+        <v>193</v>
       </c>
       <c r="C55" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="B56" t="s">
-        <v>209</v>
+        <v>195</v>
       </c>
       <c r="C56" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="B57" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="C57" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="B58" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="C58" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="B59" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="C59" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="B60" t="s">
-        <v>345</v>
+        <v>203</v>
       </c>
       <c r="C60" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B61" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="C61" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="B62" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C62" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="B63" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="C63" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="B64" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="B65" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="C65" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="B66" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="C66" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="B67" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C67" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>230</v>
+        <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>231</v>
+        <v>278</v>
       </c>
       <c r="C68" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>232</v>
+        <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>233</v>
+        <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>234</v>
+        <v>5</v>
       </c>
       <c r="B70" t="s">
-        <v>235</v>
+        <v>280</v>
       </c>
       <c r="C70" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>236</v>
+        <v>6</v>
       </c>
       <c r="B71" t="s">
-        <v>237</v>
+        <v>281</v>
       </c>
       <c r="C71" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>238</v>
+        <v>7</v>
       </c>
       <c r="B72" t="s">
-        <v>239</v>
+        <v>282</v>
       </c>
       <c r="C72" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>240</v>
+        <v>8</v>
       </c>
       <c r="B73" t="s">
-        <v>241</v>
+        <v>283</v>
       </c>
       <c r="C73" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>242</v>
+        <v>9</v>
       </c>
       <c r="B74" t="s">
-        <v>243</v>
+        <v>295</v>
       </c>
       <c r="C74" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>244</v>
+        <v>10</v>
       </c>
       <c r="B75" t="s">
-        <v>245</v>
+        <v>11</v>
       </c>
       <c r="C75" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>246</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>247</v>
+        <v>13</v>
       </c>
       <c r="C76" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>248</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>249</v>
-      </c>
-      <c r="C77" t="s">
-        <v>326</v>
+        <v>284</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>250</v>
+        <v>15</v>
       </c>
       <c r="B78" t="s">
-        <v>251</v>
+        <v>16</v>
       </c>
       <c r="C78" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B79" t="s">
-        <v>328</v>
+        <v>294</v>
       </c>
       <c r="C79" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="B80" t="s">
-        <v>4</v>
+        <v>285</v>
       </c>
       <c r="C80" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>330</v>
+        <v>286</v>
       </c>
       <c r="C81" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="B82" t="s">
-        <v>331</v>
+        <v>287</v>
       </c>
       <c r="C82" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B83" t="s">
-        <v>332</v>
+        <v>22</v>
       </c>
       <c r="C83" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="B84" t="s">
-        <v>333</v>
+        <v>24</v>
       </c>
       <c r="C84" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B85" t="s">
-        <v>334</v>
+        <v>292</v>
       </c>
       <c r="C85" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B86" t="s">
-        <v>351</v>
+        <v>293</v>
       </c>
       <c r="C86" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="B87" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="C87" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B88" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="C88" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="B89" t="s">
-        <v>336</v>
+        <v>31</v>
       </c>
       <c r="C89" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>335</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>327</v>
+        <v>33</v>
+      </c>
+      <c r="C90" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="B91" t="s">
-        <v>337</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>327</v>
+        <v>35</v>
+      </c>
+      <c r="C91" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B92" t="s">
-        <v>338</v>
+        <v>37</v>
       </c>
       <c r="C92" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B93" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C93" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B94" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="C94" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B95" t="s">
-        <v>339</v>
+        <v>43</v>
       </c>
       <c r="C95" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="B96" t="s">
-        <v>350</v>
+        <v>45</v>
       </c>
       <c r="C96" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="B97" t="s">
-        <v>340</v>
+        <v>47</v>
       </c>
       <c r="C97" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="B98" t="s">
-        <v>341</v>
+        <v>49</v>
       </c>
       <c r="C98" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B99" t="s">
-        <v>342</v>
+        <v>51</v>
       </c>
       <c r="C99" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="B100" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="C100" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="B101" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C101" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B102" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="C102" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="B103" t="s">
-        <v>348</v>
+        <v>59</v>
       </c>
       <c r="C103" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="B104" t="s">
-        <v>349</v>
+        <v>61</v>
       </c>
       <c r="C104" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="B105" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="C105" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="B106" t="s">
-        <v>38</v>
+        <v>65</v>
       </c>
       <c r="C106" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>39</v>
-      </c>
-      <c r="B107" t="s">
-        <v>40</v>
-      </c>
-      <c r="C107" t="s">
-        <v>326</v>
+      <c r="A107" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B107" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="B108" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="C108" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="B109" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="C109" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
       <c r="B110" t="s">
-        <v>46</v>
+        <v>73</v>
       </c>
       <c r="C110" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="B111" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="C111" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B112" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C112" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="B113" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="C113" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="B114" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="C114" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="B115" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="C115" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="B116" t="s">
-        <v>58</v>
+        <v>289</v>
       </c>
       <c r="C116" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="B117" t="s">
-        <v>60</v>
+        <v>291</v>
       </c>
       <c r="C117" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="B118" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="C118" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="B119" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="C119" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="B120" t="s">
-        <v>66</v>
+        <v>91</v>
       </c>
       <c r="C120" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="B121" t="s">
-        <v>68</v>
+        <v>93</v>
       </c>
       <c r="C121" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>69</v>
+        <v>94</v>
       </c>
       <c r="B122" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C122" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="B123" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="C123" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="B124" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="C124" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="B125" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="C125" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="B126" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="C126" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="B127" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="C127" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="B128" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="C128" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="B129" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="C129" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A130" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>343</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>326</v>
+      <c r="A130" t="s">
+        <v>110</v>
+      </c>
+      <c r="B130" t="s">
+        <v>111</v>
+      </c>
+      <c r="C130" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="B131" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="C131" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="B132" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="C132" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="B133" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="C133" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="B134" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="C134" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="B135" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="C135" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="B136" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="C136" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="B137" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C137" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="B138" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="C138" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="B139" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="C139" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
       <c r="B140" t="s">
-        <v>344</v>
+        <v>290</v>
       </c>
       <c r="C140" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="B141" t="s">
-        <v>347</v>
+        <v>132</v>
       </c>
       <c r="C141" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="B142" t="s">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="C142" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="B143" t="s">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="C143" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>111</v>
+        <v>137</v>
       </c>
       <c r="B144" t="s">
-        <v>112</v>
+        <v>138</v>
       </c>
       <c r="C144" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>113</v>
+        <v>139</v>
       </c>
       <c r="B145" t="s">
-        <v>114</v>
+        <v>140</v>
       </c>
       <c r="C145" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="B146" t="s">
-        <v>116</v>
+        <v>142</v>
       </c>
       <c r="C146" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>117</v>
+        <v>143</v>
       </c>
       <c r="B147" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="C147" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>119</v>
+        <v>145</v>
       </c>
       <c r="B148" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="C148" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>121</v>
+        <v>147</v>
       </c>
       <c r="B149" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
       <c r="C149" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>123</v>
+        <v>314</v>
       </c>
       <c r="B150" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="C150" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>125</v>
+        <v>313</v>
       </c>
       <c r="B151" t="s">
-        <v>126</v>
+        <v>312</v>
       </c>
       <c r="C151" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>127</v>
+        <v>311</v>
       </c>
       <c r="B152" t="s">
-        <v>128</v>
+        <v>310</v>
       </c>
       <c r="C152" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>129</v>
+        <v>309</v>
       </c>
       <c r="B153" t="s">
-        <v>130</v>
+        <v>308</v>
       </c>
       <c r="C153" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>131</v>
+        <v>307</v>
       </c>
       <c r="B154" t="s">
-        <v>132</v>
+        <v>306</v>
       </c>
       <c r="C154" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>133</v>
+        <v>305</v>
       </c>
       <c r="B155" t="s">
-        <v>134</v>
+        <v>304</v>
       </c>
       <c r="C155" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>135</v>
+        <v>303</v>
       </c>
       <c r="B156" t="s">
-        <v>136</v>
+        <v>302</v>
       </c>
       <c r="C156" t="s">
-        <v>327</v>
+        <v>276</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>137</v>
+        <v>301</v>
       </c>
       <c r="B157" t="s">
-        <v>138</v>
+        <v>300</v>
       </c>
       <c r="C157" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>139</v>
+        <v>328</v>
       </c>
       <c r="B158" t="s">
-        <v>140</v>
+        <v>327</v>
       </c>
       <c r="C158" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>141</v>
+        <v>326</v>
       </c>
       <c r="B159" t="s">
-        <v>142</v>
+        <v>325</v>
       </c>
       <c r="C159" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>143</v>
+        <v>324</v>
       </c>
       <c r="B160" t="s">
-        <v>144</v>
+        <v>323</v>
       </c>
       <c r="C160" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>145</v>
+        <v>322</v>
       </c>
       <c r="B161" t="s">
-        <v>146</v>
+        <v>321</v>
       </c>
       <c r="C161" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>147</v>
+        <v>320</v>
       </c>
       <c r="B162" t="s">
-        <v>148</v>
+        <v>319</v>
       </c>
       <c r="C162" t="s">
-        <v>326</v>
+        <v>277</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>149</v>
+        <v>318</v>
       </c>
       <c r="B163" t="s">
-        <v>150</v>
+        <v>317</v>
       </c>
       <c r="C163" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>151</v>
+        <v>316</v>
       </c>
       <c r="B164" t="s">
-        <v>152</v>
+        <v>315</v>
       </c>
       <c r="C164" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A165" t="s">
-        <v>153</v>
-      </c>
-      <c r="B165" t="s">
-        <v>346</v>
-      </c>
-      <c r="C165" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A166" t="s">
-        <v>154</v>
-      </c>
-      <c r="B166" t="s">
-        <v>155</v>
-      </c>
-      <c r="C166" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A167" t="s">
-        <v>156</v>
-      </c>
-      <c r="B167" t="s">
-        <v>157</v>
-      </c>
-      <c r="C167" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A168" t="s">
-        <v>158</v>
-      </c>
-      <c r="B168" t="s">
-        <v>159</v>
-      </c>
-      <c r="C168" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A169" t="s">
-        <v>160</v>
-      </c>
-      <c r="B169" t="s">
-        <v>161</v>
-      </c>
-      <c r="C169" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A170" t="s">
-        <v>162</v>
-      </c>
-      <c r="B170" t="s">
-        <v>163</v>
-      </c>
-      <c r="C170" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A171" t="s">
-        <v>164</v>
-      </c>
-      <c r="B171" t="s">
-        <v>165</v>
-      </c>
-      <c r="C171" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A172" t="s">
-        <v>166</v>
-      </c>
-      <c r="B172" t="s">
-        <v>167</v>
-      </c>
-      <c r="C172" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>168</v>
-      </c>
-      <c r="B173" t="s">
-        <v>169</v>
-      </c>
-      <c r="C173" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A174" t="s">
-        <v>170</v>
-      </c>
-      <c r="B174" t="s">
-        <v>171</v>
-      </c>
-      <c r="C174" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A175" t="s">
-        <v>172</v>
-      </c>
-      <c r="B175" t="s">
-        <v>173</v>
-      </c>
-      <c r="C175" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A176" t="s">
-        <v>174</v>
-      </c>
-      <c r="B176" t="s">
-        <v>175</v>
-      </c>
-      <c r="C176" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A177" t="s">
-        <v>176</v>
-      </c>
-      <c r="B177" t="s">
-        <v>177</v>
-      </c>
-      <c r="C177" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A178" t="s">
-        <v>378</v>
-      </c>
-      <c r="B178" t="s">
-        <v>377</v>
-      </c>
-      <c r="C178" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A179" t="s">
-        <v>376</v>
-      </c>
-      <c r="B179" t="s">
-        <v>163</v>
-      </c>
-      <c r="C179" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
-        <v>375</v>
-      </c>
-      <c r="B180" t="s">
-        <v>374</v>
-      </c>
-      <c r="C180" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>373</v>
-      </c>
-      <c r="B181" t="s">
-        <v>372</v>
-      </c>
-      <c r="C181" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
-        <v>371</v>
-      </c>
-      <c r="B182" t="s">
-        <v>370</v>
-      </c>
-      <c r="C182" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
-        <v>369</v>
-      </c>
-      <c r="B183" t="s">
-        <v>368</v>
-      </c>
-      <c r="C183" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
-        <v>367</v>
-      </c>
-      <c r="B184" t="s">
-        <v>366</v>
-      </c>
-      <c r="C184" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A185" t="s">
-        <v>365</v>
-      </c>
-      <c r="B185" t="s">
-        <v>364</v>
-      </c>
-      <c r="C185" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A186" t="s">
-        <v>363</v>
-      </c>
-      <c r="B186" t="s">
-        <v>362</v>
-      </c>
-      <c r="C186" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A187" t="s">
-        <v>361</v>
-      </c>
-      <c r="B187" t="s">
-        <v>360</v>
-      </c>
-      <c r="C187" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A188" t="s">
-        <v>359</v>
-      </c>
-      <c r="B188" t="s">
-        <v>358</v>
-      </c>
-      <c r="C188" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
-        <v>356</v>
-      </c>
-      <c r="B189" t="s">
-        <v>357</v>
-      </c>
-      <c r="C189" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A190" t="s">
-        <v>394</v>
-      </c>
-      <c r="B190" t="s">
-        <v>393</v>
-      </c>
-      <c r="C190" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A191" t="s">
-        <v>392</v>
-      </c>
-      <c r="B191" t="s">
-        <v>391</v>
-      </c>
-      <c r="C191" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A192" t="s">
-        <v>390</v>
-      </c>
-      <c r="B192" t="s">
-        <v>389</v>
-      </c>
-      <c r="C192" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A193" t="s">
-        <v>388</v>
-      </c>
-      <c r="B193" t="s">
-        <v>387</v>
-      </c>
-      <c r="C193" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A194" t="s">
-        <v>386</v>
-      </c>
-      <c r="B194" t="s">
-        <v>385</v>
-      </c>
-      <c r="C194" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A195" t="s">
-        <v>384</v>
-      </c>
-      <c r="B195" t="s">
-        <v>383</v>
-      </c>
-      <c r="C195" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A196" t="s">
-        <v>382</v>
-      </c>
-      <c r="B196" t="s">
-        <v>381</v>
-      </c>
-      <c r="C196" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A197" t="s">
-        <v>380</v>
-      </c>
-      <c r="B197" t="s">
-        <v>379</v>
-      </c>
-      <c r="C197" t="s">
-        <v>327</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Jobs - 4 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B15212CD-8CAC-437C-AB06-F3738C8EB622}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACD6A732-98E4-4CE5-B221-B716FD9955FA}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="367">
   <si>
     <t>Job</t>
   </si>
@@ -1098,6 +1098,48 @@
   </si>
   <si>
     <t>1085291 - 00059958 - DG Label</t>
+  </si>
+  <si>
+    <t>1085378 - 00050724 - DG Label</t>
+  </si>
+  <si>
+    <t>51A Southdown Drive, Martinborough</t>
+  </si>
+  <si>
+    <t>1085377 - 00052076 - DG Label</t>
+  </si>
+  <si>
+    <t>8C Michael Street, Masterton</t>
+  </si>
+  <si>
+    <t>1085376 - 00064756 - DG Label</t>
+  </si>
+  <si>
+    <t>6A Garrity Lane, Greytown</t>
+  </si>
+  <si>
+    <t>1085373 - 00037564 - DG Label</t>
+  </si>
+  <si>
+    <t>41 Kowhai Street, Castelcliff</t>
+  </si>
+  <si>
+    <t>1085371 - 00053149 - DG Label</t>
+  </si>
+  <si>
+    <t>56 Willoughby Street, Halcombe</t>
+  </si>
+  <si>
+    <t>1085370 - 00061230 - DG Label</t>
+  </si>
+  <si>
+    <t>130 Mount Biggs Road, Halcombe</t>
+  </si>
+  <si>
+    <t>1085369 - 00053697 - DG Label</t>
+  </si>
+  <si>
+    <t>121 Taikorea Road, Glen Oroua</t>
   </si>
 </sst>
 </file>
@@ -1478,7 +1520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C176"/>
+  <dimension ref="A1:C183"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -3422,6 +3464,83 @@
         <v>276</v>
       </c>
     </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>353</v>
+      </c>
+      <c r="B177" t="s">
+        <v>354</v>
+      </c>
+      <c r="C177" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>355</v>
+      </c>
+      <c r="B178" t="s">
+        <v>356</v>
+      </c>
+      <c r="C178" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>357</v>
+      </c>
+      <c r="B179" t="s">
+        <v>358</v>
+      </c>
+      <c r="C179" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>359</v>
+      </c>
+      <c r="B180" t="s">
+        <v>360</v>
+      </c>
+      <c r="C180" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>361</v>
+      </c>
+      <c r="B181" t="s">
+        <v>362</v>
+      </c>
+      <c r="C181" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>363</v>
+      </c>
+      <c r="B182" t="s">
+        <v>364</v>
+      </c>
+      <c r="C182" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>365</v>
+      </c>
+      <c r="B183" t="s">
+        <v>366</v>
+      </c>
+      <c r="C183" t="s">
+        <v>276</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Removed completed Jobs 4 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACD6A732-98E4-4CE5-B221-B716FD9955FA}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE64BFAB-F577-4249-A9EA-FF99EB5F363D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="359">
   <si>
     <t>Job</t>
   </si>
@@ -68,9 +68,6 @@
     <t>1084461 - 00050984 - DG Label</t>
   </si>
   <si>
-    <t>1084460 - 00053371 - DG Label</t>
-  </si>
-  <si>
     <t>1084307 - 00059085 - DG Label</t>
   </si>
   <si>
@@ -383,12 +380,6 @@
     <t>142A Dublin Street, Martinborough</t>
   </si>
   <si>
-    <t>1083505 - 00056798 - DG Label</t>
-  </si>
-  <si>
-    <t>12 Campbell Drive, Martinborough</t>
-  </si>
-  <si>
     <t>1083503 - 00055234 - DG Label</t>
   </si>
   <si>
@@ -497,12 +488,6 @@
     <t>56 FREDERICK ST, CARTERTON</t>
   </si>
   <si>
-    <t>1082790 - 00033944 - DG Label</t>
-  </si>
-  <si>
-    <t>214A Dry River Road, Dyerville</t>
-  </si>
-  <si>
     <t>1082789 - 00029633 - DG Label</t>
   </si>
   <si>
@@ -641,12 +626,6 @@
     <t>11 Moore Street, Featherston</t>
   </si>
   <si>
-    <t>1081143 - 00042916 - DG Label</t>
-  </si>
-  <si>
-    <t>12 Cherry Lane, Martinborough</t>
-  </si>
-  <si>
     <t>1081142 - 00042583 - DG Label</t>
   </si>
   <si>
@@ -924,9 +903,6 @@
   </si>
   <si>
     <t>3 Paterson Lane, Kelvin Grove</t>
-  </si>
-  <si>
-    <t>26 Romina Way, Martinborough</t>
   </si>
   <si>
     <t>Nga Waka Winery, Martinborough</t>
@@ -1520,7 +1496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C183"/>
+  <dimension ref="A1:C179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -1536,1932 +1512,1932 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C2" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B3" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="B4" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C4" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B5" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C5" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C6" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B7" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="C7" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B8" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C8" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B9" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C9" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B10" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C10" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B11" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C11" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B12" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C12" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B13" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C13" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="B14" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="C14" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B15" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="C15" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B16" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="C16" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="B17" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C17" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="B18" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C18" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="B19" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C19" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="B20" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C20" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B21" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="C21" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="B22" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="C22" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B23" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C23" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="B24" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C24" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="B25" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="C25" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="B26" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="C26" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B27" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C27" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="B28" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="C28" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B29" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C29" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B30" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="C30" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B31" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="C31" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B32" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="C32" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B33" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C33" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B34" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C34" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B35" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C35" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B36" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C36" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B37" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C37" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B38" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B39" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C39" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B40" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B41" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C41" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B42" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B43" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C43" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B44" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B45" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C45" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B46" t="s">
-        <v>177</v>
+        <v>288</v>
       </c>
       <c r="C46" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B47" t="s">
-        <v>296</v>
+        <v>175</v>
       </c>
       <c r="C47" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B48" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C48" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B49" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C49" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B50" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C50" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B51" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C51" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B52" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C52" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B53" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C53" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B54" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C54" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B55" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C55" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B56" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C56" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B57" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C57" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B58" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C58" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B60" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C60" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B61" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C61" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B62" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C62" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B63" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C63" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B64" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C64" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B65" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C65" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>214</v>
+        <v>2</v>
       </c>
       <c r="B66" t="s">
-        <v>215</v>
+        <v>271</v>
       </c>
       <c r="C66" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>216</v>
+        <v>3</v>
       </c>
       <c r="B67" t="s">
-        <v>217</v>
+        <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B68" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C68" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B69" t="s">
-        <v>4</v>
+        <v>274</v>
       </c>
       <c r="C69" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B70" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C70" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B71" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="C71" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B72" t="s">
-        <v>282</v>
+        <v>10</v>
       </c>
       <c r="C72" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>283</v>
+        <v>12</v>
       </c>
       <c r="C73" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B74" t="s">
-        <v>295</v>
-      </c>
-      <c r="C74" t="s">
         <v>277</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B75" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C75" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B76" t="s">
-        <v>13</v>
+        <v>287</v>
       </c>
       <c r="C76" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B77" t="s">
-        <v>284</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
+      </c>
+      <c r="C77" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B78" t="s">
-        <v>16</v>
+        <v>279</v>
       </c>
       <c r="C78" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="C79" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B80" t="s">
-        <v>285</v>
+        <v>21</v>
       </c>
       <c r="C80" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B81" t="s">
-        <v>286</v>
+        <v>23</v>
       </c>
       <c r="C81" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B82" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C82" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B83" t="s">
-        <v>22</v>
+        <v>286</v>
       </c>
       <c r="C83" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="B84" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="C84" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B85" t="s">
-        <v>292</v>
+        <v>28</v>
       </c>
       <c r="C85" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B86" t="s">
-        <v>293</v>
+        <v>30</v>
       </c>
       <c r="C86" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="B87" t="s">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="C87" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B88" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C88" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B89" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C89" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B90" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C90" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B92" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C92" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B93" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C93" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B94" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C94" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B95" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C95" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B96" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C96" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B97" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C97" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B98" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C98" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B99" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C99" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B100" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C100" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B101" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C101" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B102" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C102" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B103" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C103" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>60</v>
-      </c>
-      <c r="B104" t="s">
-        <v>61</v>
-      </c>
-      <c r="C104" t="s">
-        <v>277</v>
+      <c r="A104" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B105" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B106" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C106" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A107" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>276</v>
+      <c r="A107" t="s">
+        <v>71</v>
+      </c>
+      <c r="B107" t="s">
+        <v>72</v>
+      </c>
+      <c r="C107" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B108" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C108" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B109" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C109" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B110" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C110" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B111" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C111" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B112" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C112" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B113" t="s">
-        <v>79</v>
+        <v>282</v>
       </c>
       <c r="C113" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B114" t="s">
-        <v>81</v>
+        <v>284</v>
       </c>
       <c r="C114" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B115" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C115" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B116" t="s">
-        <v>289</v>
+        <v>88</v>
       </c>
       <c r="C116" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B117" t="s">
-        <v>291</v>
+        <v>90</v>
       </c>
       <c r="C117" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B118" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C118" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B119" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C119" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B120" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C120" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B121" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C121" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B122" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C122" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B123" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C123" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B124" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C124" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B125" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C125" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B126" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C126" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B127" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C127" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B128" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C128" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B129" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C129" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B130" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C130" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B131" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="C131" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B132" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C132" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B133" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C133" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B134" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C134" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B135" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C135" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B136" t="s">
-        <v>123</v>
+        <v>283</v>
       </c>
       <c r="C136" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B137" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C137" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B138" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C138" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B139" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C139" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B140" t="s">
-        <v>290</v>
+        <v>135</v>
       </c>
       <c r="C140" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B141" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C141" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B142" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C142" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B143" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C143" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B144" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C144" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C145" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>141</v>
+        <v>306</v>
       </c>
       <c r="B146" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C146" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>143</v>
+        <v>305</v>
       </c>
       <c r="B147" t="s">
-        <v>144</v>
+        <v>304</v>
       </c>
       <c r="C147" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>145</v>
+        <v>303</v>
       </c>
       <c r="B148" t="s">
-        <v>146</v>
+        <v>302</v>
       </c>
       <c r="C148" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>147</v>
+        <v>301</v>
       </c>
       <c r="B149" t="s">
-        <v>148</v>
+        <v>300</v>
       </c>
       <c r="C149" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="B150" t="s">
-        <v>138</v>
+        <v>298</v>
       </c>
       <c r="C150" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>313</v>
+        <v>297</v>
       </c>
       <c r="B151" t="s">
-        <v>312</v>
+        <v>296</v>
       </c>
       <c r="C151" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>311</v>
+        <v>295</v>
       </c>
       <c r="B152" t="s">
-        <v>310</v>
+        <v>294</v>
       </c>
       <c r="C152" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="B153" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="C153" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="B154" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
       <c r="C154" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="B155" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="C155" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="B156" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="C156" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="B157" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="C157" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="B158" t="s">
-        <v>327</v>
+        <v>311</v>
       </c>
       <c r="C158" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>326</v>
+        <v>310</v>
       </c>
       <c r="B159" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="C159" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>324</v>
+        <v>308</v>
       </c>
       <c r="B160" t="s">
-        <v>323</v>
+        <v>307</v>
       </c>
       <c r="C160" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>322</v>
+        <v>344</v>
       </c>
       <c r="B161" t="s">
-        <v>321</v>
+        <v>343</v>
       </c>
       <c r="C161" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>320</v>
+        <v>342</v>
       </c>
       <c r="B162" t="s">
-        <v>319</v>
+        <v>341</v>
       </c>
       <c r="C162" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>318</v>
+        <v>340</v>
       </c>
       <c r="B163" t="s">
-        <v>317</v>
+        <v>339</v>
       </c>
       <c r="C163" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>316</v>
+        <v>338</v>
       </c>
       <c r="B164" t="s">
-        <v>315</v>
+        <v>337</v>
       </c>
       <c r="C164" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>352</v>
+        <v>336</v>
       </c>
       <c r="B165" t="s">
-        <v>351</v>
+        <v>335</v>
       </c>
       <c r="C165" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="B166" t="s">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="C166" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>348</v>
+        <v>332</v>
       </c>
       <c r="B167" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
       <c r="C167" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="B168" t="s">
-        <v>345</v>
+        <v>329</v>
       </c>
       <c r="C168" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>344</v>
+        <v>328</v>
       </c>
       <c r="B169" t="s">
-        <v>343</v>
+        <v>327</v>
       </c>
       <c r="C169" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>342</v>
+        <v>326</v>
       </c>
       <c r="B170" t="s">
-        <v>341</v>
+        <v>325</v>
       </c>
       <c r="C170" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>340</v>
+        <v>324</v>
       </c>
       <c r="B171" t="s">
-        <v>339</v>
+        <v>323</v>
       </c>
       <c r="C171" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>338</v>
+        <v>322</v>
       </c>
       <c r="B172" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="C172" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="B173" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="C173" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
       <c r="B174" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="C174" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>332</v>
+        <v>349</v>
       </c>
       <c r="B175" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="C175" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>330</v>
+        <v>351</v>
       </c>
       <c r="B176" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="C176" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -3472,7 +3448,7 @@
         <v>354</v>
       </c>
       <c r="C177" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -3483,7 +3459,7 @@
         <v>356</v>
       </c>
       <c r="C178" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -3494,51 +3470,7 @@
         <v>358</v>
       </c>
       <c r="C179" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A180" t="s">
-        <v>359</v>
-      </c>
-      <c r="B180" t="s">
-        <v>360</v>
-      </c>
-      <c r="C180" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A181" t="s">
-        <v>361</v>
-      </c>
-      <c r="B181" t="s">
-        <v>362</v>
-      </c>
-      <c r="C181" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A182" t="s">
-        <v>363</v>
-      </c>
-      <c r="B182" t="s">
-        <v>364</v>
-      </c>
-      <c r="C182" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A183" t="s">
-        <v>365</v>
-      </c>
-      <c r="B183" t="s">
-        <v>366</v>
-      </c>
-      <c r="C183" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new jobs and added process 4 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE64BFAB-F577-4249-A9EA-FF99EB5F363D}"/>
+  <xr:revisionPtr revIDLastSave="118" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA7284FF-052E-471C-B7A7-A8973B5C7845}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="365">
   <si>
     <t>Job</t>
   </si>
@@ -1116,6 +1116,24 @@
   </si>
   <si>
     <t>121 Taikorea Road, Glen Oroua</t>
+  </si>
+  <si>
+    <t>1085457 - 00055046 - DG Label</t>
+  </si>
+  <si>
+    <t>63 Otawa Drive, Carterton</t>
+  </si>
+  <si>
+    <t>1085460 - 00026995 - DG Label</t>
+  </si>
+  <si>
+    <t>73 Young Street, Whanganui East</t>
+  </si>
+  <si>
+    <t>1085458 - 00044870 - DG Label</t>
+  </si>
+  <si>
+    <t>70B Duddings Lane, Featherson</t>
   </si>
 </sst>
 </file>
@@ -1496,7 +1514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C179"/>
+  <dimension ref="A1:C182"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -3473,6 +3491,39 @@
         <v>269</v>
       </c>
     </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>359</v>
+      </c>
+      <c r="B180" t="s">
+        <v>360</v>
+      </c>
+      <c r="C180" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>361</v>
+      </c>
+      <c r="B181" t="s">
+        <v>362</v>
+      </c>
+      <c r="C181" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>363</v>
+      </c>
+      <c r="B182" t="s">
+        <v>364</v>
+      </c>
+      <c r="C182" t="s">
+        <v>270</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added jobs 5 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA7284FF-052E-471C-B7A7-A8973B5C7845}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D751C798-9842-41FC-9857-15A61752D38E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="383">
   <si>
     <t>Job</t>
   </si>
@@ -1134,13 +1134,67 @@
   </si>
   <si>
     <t>70B Duddings Lane, Featherson</t>
+  </si>
+  <si>
+    <t>1085533 - 00050342 - DG Label</t>
+  </si>
+  <si>
+    <t>25 Whisky Way, Aokautere</t>
+  </si>
+  <si>
+    <t>1085531 - 00056810 - DG Label</t>
+  </si>
+  <si>
+    <t>289A Fabians Road, Greytown</t>
+  </si>
+  <si>
+    <t>1085529 - 00052073 - DG Label</t>
+  </si>
+  <si>
+    <t>1 Valkyrie Close, Carterton</t>
+  </si>
+  <si>
+    <t>1085528 - 00052070 - DG Label</t>
+  </si>
+  <si>
+    <t>72 Jellicoe Street, Greytown</t>
+  </si>
+  <si>
+    <t>1085526 - 00052065 - DG Label</t>
+  </si>
+  <si>
+    <t>966 Kahutara Road, Kahutara</t>
+  </si>
+  <si>
+    <t>1085525 - 00050727 - DG Label</t>
+  </si>
+  <si>
+    <t>138 Loop Line, Opaki</t>
+  </si>
+  <si>
+    <t>1085524 - 00050503 - DG Label</t>
+  </si>
+  <si>
+    <t>29 Harrison Street West, Featherston</t>
+  </si>
+  <si>
+    <t>1085522 - 00050476 - DG Label</t>
+  </si>
+  <si>
+    <t>194 Kiriwhakapapa Road, Masterton</t>
+  </si>
+  <si>
+    <t>1085521 - 00048180 - DG Label</t>
+  </si>
+  <si>
+    <t>49 Wards Line, Greytown</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1514,15 +1568,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C182"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C191"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1533,7 +1587,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>211</v>
       </c>
@@ -1544,7 +1598,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>213</v>
       </c>
@@ -1555,7 +1609,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>215</v>
       </c>
@@ -1566,7 +1620,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>217</v>
       </c>
@@ -1577,7 +1631,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>219</v>
       </c>
@@ -1588,7 +1642,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>221</v>
       </c>
@@ -1599,7 +1653,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>223</v>
       </c>
@@ -1610,7 +1664,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>225</v>
       </c>
@@ -1621,7 +1675,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>227</v>
       </c>
@@ -1632,7 +1686,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>229</v>
       </c>
@@ -1643,7 +1697,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>231</v>
       </c>
@@ -1654,7 +1708,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>233</v>
       </c>
@@ -1665,7 +1719,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>235</v>
       </c>
@@ -1676,7 +1730,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>237</v>
       </c>
@@ -1687,7 +1741,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>239</v>
       </c>
@@ -1698,7 +1752,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>241</v>
       </c>
@@ -1709,7 +1763,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>243</v>
       </c>
@@ -1720,7 +1774,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>245</v>
       </c>
@@ -1731,7 +1785,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>247</v>
       </c>
@@ -1742,7 +1796,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>249</v>
       </c>
@@ -1753,7 +1807,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>251</v>
       </c>
@@ -1764,7 +1818,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>253</v>
       </c>
@@ -1775,7 +1829,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>255</v>
       </c>
@@ -1786,7 +1840,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>257</v>
       </c>
@@ -1797,7 +1851,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" t="s">
         <v>259</v>
       </c>
@@ -1808,7 +1862,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3">
       <c r="A27" t="s">
         <v>260</v>
       </c>
@@ -1819,7 +1873,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>262</v>
       </c>
@@ -1830,7 +1884,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>264</v>
       </c>
@@ -1841,7 +1895,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3">
       <c r="A30" t="s">
         <v>266</v>
       </c>
@@ -1852,7 +1906,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3">
       <c r="A31" t="s">
         <v>268</v>
       </c>
@@ -1863,7 +1917,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32" t="s">
         <v>146</v>
       </c>
@@ -1874,7 +1928,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>147</v>
       </c>
@@ -1885,7 +1939,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3">
       <c r="A34" t="s">
         <v>149</v>
       </c>
@@ -1896,7 +1950,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>151</v>
       </c>
@@ -1907,7 +1961,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3">
       <c r="A36" t="s">
         <v>153</v>
       </c>
@@ -1918,7 +1972,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3">
       <c r="A37" t="s">
         <v>155</v>
       </c>
@@ -1929,7 +1983,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>157</v>
       </c>
@@ -1940,7 +1994,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3">
       <c r="A39" t="s">
         <v>159</v>
       </c>
@@ -1951,7 +2005,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -1962,7 +2016,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3">
       <c r="A41" t="s">
         <v>163</v>
       </c>
@@ -1973,7 +2027,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3">
       <c r="A42" t="s">
         <v>165</v>
       </c>
@@ -1984,7 +2038,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3">
       <c r="A43" t="s">
         <v>167</v>
       </c>
@@ -1995,7 +2049,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3">
       <c r="A44" t="s">
         <v>169</v>
       </c>
@@ -2006,7 +2060,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3">
       <c r="A45" t="s">
         <v>171</v>
       </c>
@@ -2017,7 +2071,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3">
       <c r="A46" t="s">
         <v>173</v>
       </c>
@@ -2028,7 +2082,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3">
       <c r="A47" t="s">
         <v>174</v>
       </c>
@@ -2039,7 +2093,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3">
       <c r="A48" t="s">
         <v>176</v>
       </c>
@@ -2050,7 +2104,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3">
       <c r="A49" t="s">
         <v>178</v>
       </c>
@@ -2061,7 +2115,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3">
       <c r="A50" t="s">
         <v>180</v>
       </c>
@@ -2072,7 +2126,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3">
       <c r="A51" t="s">
         <v>181</v>
       </c>
@@ -2083,7 +2137,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3">
       <c r="A52" t="s">
         <v>183</v>
       </c>
@@ -2094,7 +2148,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3">
       <c r="A53" t="s">
         <v>185</v>
       </c>
@@ -2105,7 +2159,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3">
       <c r="A54" t="s">
         <v>187</v>
       </c>
@@ -2116,7 +2170,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3">
       <c r="A55" t="s">
         <v>189</v>
       </c>
@@ -2127,7 +2181,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3">
       <c r="A56" t="s">
         <v>191</v>
       </c>
@@ -2138,7 +2192,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3">
       <c r="A57" t="s">
         <v>193</v>
       </c>
@@ -2149,7 +2203,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3">
       <c r="A58" t="s">
         <v>195</v>
       </c>
@@ -2160,7 +2214,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3">
       <c r="A59" t="s">
         <v>197</v>
       </c>
@@ -2171,7 +2225,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3">
       <c r="A60" t="s">
         <v>199</v>
       </c>
@@ -2182,7 +2236,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3">
       <c r="A61" t="s">
         <v>201</v>
       </c>
@@ -2193,7 +2247,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3">
       <c r="A62" t="s">
         <v>203</v>
       </c>
@@ -2204,7 +2258,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3">
       <c r="A63" t="s">
         <v>205</v>
       </c>
@@ -2215,7 +2269,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3">
       <c r="A64" t="s">
         <v>207</v>
       </c>
@@ -2226,7 +2280,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3">
       <c r="A65" t="s">
         <v>209</v>
       </c>
@@ -2237,7 +2291,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2248,7 +2302,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -2259,7 +2313,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3">
       <c r="A68" t="s">
         <v>5</v>
       </c>
@@ -2270,7 +2324,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3">
       <c r="A69" t="s">
         <v>6</v>
       </c>
@@ -2281,7 +2335,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3">
       <c r="A70" t="s">
         <v>7</v>
       </c>
@@ -2292,7 +2346,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -2303,7 +2357,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -2314,7 +2368,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2325,7 +2379,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -2336,7 +2390,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3">
       <c r="A75" t="s">
         <v>14</v>
       </c>
@@ -2347,7 +2401,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -2358,7 +2412,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3">
       <c r="A77" t="s">
         <v>17</v>
       </c>
@@ -2369,7 +2423,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3">
       <c r="A78" t="s">
         <v>18</v>
       </c>
@@ -2380,7 +2434,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3">
       <c r="A79" t="s">
         <v>19</v>
       </c>
@@ -2391,7 +2445,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3">
       <c r="A80" t="s">
         <v>20</v>
       </c>
@@ -2402,7 +2456,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3">
       <c r="A81" t="s">
         <v>22</v>
       </c>
@@ -2413,7 +2467,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3">
       <c r="A82" t="s">
         <v>24</v>
       </c>
@@ -2424,7 +2478,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3">
       <c r="A83" t="s">
         <v>25</v>
       </c>
@@ -2435,7 +2489,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3">
       <c r="A84" t="s">
         <v>65</v>
       </c>
@@ -2446,7 +2500,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -2457,7 +2511,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3">
       <c r="A86" t="s">
         <v>29</v>
       </c>
@@ -2468,7 +2522,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3">
       <c r="A87" t="s">
         <v>31</v>
       </c>
@@ -2479,7 +2533,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3">
       <c r="A88" t="s">
         <v>33</v>
       </c>
@@ -2490,7 +2544,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3">
       <c r="A89" t="s">
         <v>35</v>
       </c>
@@ -2501,7 +2555,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3">
       <c r="A90" t="s">
         <v>37</v>
       </c>
@@ -2512,7 +2566,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3">
       <c r="A91" t="s">
         <v>39</v>
       </c>
@@ -2523,7 +2577,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3">
       <c r="A92" t="s">
         <v>41</v>
       </c>
@@ -2534,7 +2588,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3">
       <c r="A93" t="s">
         <v>43</v>
       </c>
@@ -2545,7 +2599,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3">
       <c r="A94" t="s">
         <v>45</v>
       </c>
@@ -2556,7 +2610,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3">
       <c r="A95" t="s">
         <v>47</v>
       </c>
@@ -2567,7 +2621,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3">
       <c r="A96" t="s">
         <v>49</v>
       </c>
@@ -2578,7 +2632,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3">
       <c r="A97" t="s">
         <v>51</v>
       </c>
@@ -2589,7 +2643,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3">
       <c r="A98" t="s">
         <v>53</v>
       </c>
@@ -2600,7 +2654,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3">
       <c r="A99" t="s">
         <v>55</v>
       </c>
@@ -2611,7 +2665,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3">
       <c r="A100" t="s">
         <v>57</v>
       </c>
@@ -2622,7 +2676,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3">
       <c r="A101" t="s">
         <v>59</v>
       </c>
@@ -2633,7 +2687,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3">
       <c r="A102" t="s">
         <v>61</v>
       </c>
@@ -2644,7 +2698,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3">
       <c r="A103" t="s">
         <v>63</v>
       </c>
@@ -2655,7 +2709,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3">
       <c r="A104" s="2" t="s">
         <v>26</v>
       </c>
@@ -2666,7 +2720,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3">
       <c r="A105" t="s">
         <v>67</v>
       </c>
@@ -2677,7 +2731,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3">
       <c r="A106" t="s">
         <v>69</v>
       </c>
@@ -2688,7 +2742,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3">
       <c r="A107" t="s">
         <v>71</v>
       </c>
@@ -2699,7 +2753,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3">
       <c r="A108" t="s">
         <v>73</v>
       </c>
@@ -2710,7 +2764,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3">
       <c r="A109" t="s">
         <v>75</v>
       </c>
@@ -2721,7 +2775,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3">
       <c r="A110" t="s">
         <v>77</v>
       </c>
@@ -2732,7 +2786,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3">
       <c r="A111" t="s">
         <v>79</v>
       </c>
@@ -2743,7 +2797,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3">
       <c r="A112" t="s">
         <v>81</v>
       </c>
@@ -2754,7 +2808,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3">
       <c r="A113" t="s">
         <v>83</v>
       </c>
@@ -2765,7 +2819,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3">
       <c r="A114" t="s">
         <v>84</v>
       </c>
@@ -2776,7 +2830,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3">
       <c r="A115" t="s">
         <v>85</v>
       </c>
@@ -2787,7 +2841,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3">
       <c r="A116" t="s">
         <v>87</v>
       </c>
@@ -2798,7 +2852,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3">
       <c r="A117" t="s">
         <v>89</v>
       </c>
@@ -2809,7 +2863,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -2820,7 +2874,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3">
       <c r="A119" t="s">
         <v>93</v>
       </c>
@@ -2831,7 +2885,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3">
       <c r="A120" t="s">
         <v>95</v>
       </c>
@@ -2842,7 +2896,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3">
       <c r="A121" t="s">
         <v>97</v>
       </c>
@@ -2853,7 +2907,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3">
       <c r="A122" t="s">
         <v>99</v>
       </c>
@@ -2864,7 +2918,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3">
       <c r="A123" t="s">
         <v>101</v>
       </c>
@@ -2875,7 +2929,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3">
       <c r="A124" t="s">
         <v>103</v>
       </c>
@@ -2886,7 +2940,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3">
       <c r="A125" t="s">
         <v>105</v>
       </c>
@@ -2897,7 +2951,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3">
       <c r="A126" t="s">
         <v>107</v>
       </c>
@@ -2908,7 +2962,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3">
       <c r="A127" t="s">
         <v>109</v>
       </c>
@@ -2919,7 +2973,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3">
       <c r="A128" t="s">
         <v>111</v>
       </c>
@@ -2930,7 +2984,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3">
       <c r="A129" t="s">
         <v>113</v>
       </c>
@@ -2941,7 +2995,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3">
       <c r="A130" t="s">
         <v>115</v>
       </c>
@@ -2952,7 +3006,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3">
       <c r="A131" t="s">
         <v>117</v>
       </c>
@@ -2963,7 +3017,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3">
       <c r="A132" t="s">
         <v>119</v>
       </c>
@@ -2974,7 +3028,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3">
       <c r="A133" t="s">
         <v>121</v>
       </c>
@@ -2985,7 +3039,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3">
       <c r="A134" t="s">
         <v>123</v>
       </c>
@@ -2996,7 +3050,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3">
       <c r="A135" t="s">
         <v>125</v>
       </c>
@@ -3007,7 +3061,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3">
       <c r="A136" t="s">
         <v>127</v>
       </c>
@@ -3018,7 +3072,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3">
       <c r="A137" t="s">
         <v>128</v>
       </c>
@@ -3029,7 +3083,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3">
       <c r="A138" t="s">
         <v>130</v>
       </c>
@@ -3040,7 +3094,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3">
       <c r="A139" t="s">
         <v>132</v>
       </c>
@@ -3051,7 +3105,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3">
       <c r="A140" t="s">
         <v>134</v>
       </c>
@@ -3062,7 +3116,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3">
       <c r="A141" t="s">
         <v>136</v>
       </c>
@@ -3073,7 +3127,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3">
       <c r="A142" t="s">
         <v>138</v>
       </c>
@@ -3084,7 +3138,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3">
       <c r="A143" t="s">
         <v>140</v>
       </c>
@@ -3095,7 +3149,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3">
       <c r="A144" t="s">
         <v>142</v>
       </c>
@@ -3106,7 +3160,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3">
       <c r="A145" t="s">
         <v>144</v>
       </c>
@@ -3117,7 +3171,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3">
       <c r="A146" t="s">
         <v>306</v>
       </c>
@@ -3128,7 +3182,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3">
       <c r="A147" t="s">
         <v>305</v>
       </c>
@@ -3139,7 +3193,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3">
       <c r="A148" t="s">
         <v>303</v>
       </c>
@@ -3150,7 +3204,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3">
       <c r="A149" t="s">
         <v>301</v>
       </c>
@@ -3161,7 +3215,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3">
       <c r="A150" t="s">
         <v>299</v>
       </c>
@@ -3172,7 +3226,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3">
       <c r="A151" t="s">
         <v>297</v>
       </c>
@@ -3183,7 +3237,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3">
       <c r="A152" t="s">
         <v>295</v>
       </c>
@@ -3194,7 +3248,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3">
       <c r="A153" t="s">
         <v>293</v>
       </c>
@@ -3205,7 +3259,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3">
       <c r="A154" t="s">
         <v>320</v>
       </c>
@@ -3216,7 +3270,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3">
       <c r="A155" t="s">
         <v>318</v>
       </c>
@@ -3227,7 +3281,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3">
       <c r="A156" t="s">
         <v>316</v>
       </c>
@@ -3238,7 +3292,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3">
       <c r="A157" t="s">
         <v>314</v>
       </c>
@@ -3249,7 +3303,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3">
       <c r="A158" t="s">
         <v>312</v>
       </c>
@@ -3260,7 +3314,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3">
       <c r="A159" t="s">
         <v>310</v>
       </c>
@@ -3271,7 +3325,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3">
       <c r="A160" t="s">
         <v>308</v>
       </c>
@@ -3282,7 +3336,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3">
       <c r="A161" t="s">
         <v>344</v>
       </c>
@@ -3293,7 +3347,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3">
       <c r="A162" t="s">
         <v>342</v>
       </c>
@@ -3304,7 +3358,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3">
       <c r="A163" t="s">
         <v>340</v>
       </c>
@@ -3315,7 +3369,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3">
       <c r="A164" t="s">
         <v>338</v>
       </c>
@@ -3326,7 +3380,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3">
       <c r="A165" t="s">
         <v>336</v>
       </c>
@@ -3337,7 +3391,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3">
       <c r="A166" t="s">
         <v>334</v>
       </c>
@@ -3348,7 +3402,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3">
       <c r="A167" t="s">
         <v>332</v>
       </c>
@@ -3359,7 +3413,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3">
       <c r="A168" t="s">
         <v>330</v>
       </c>
@@ -3370,7 +3424,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3">
       <c r="A169" t="s">
         <v>328</v>
       </c>
@@ -3381,7 +3435,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3">
       <c r="A170" t="s">
         <v>326</v>
       </c>
@@ -3392,7 +3446,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3">
       <c r="A171" t="s">
         <v>324</v>
       </c>
@@ -3403,7 +3457,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3">
       <c r="A172" t="s">
         <v>322</v>
       </c>
@@ -3414,7 +3468,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3">
       <c r="A173" t="s">
         <v>345</v>
       </c>
@@ -3425,7 +3479,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3">
       <c r="A174" t="s">
         <v>347</v>
       </c>
@@ -3436,7 +3490,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3">
       <c r="A175" t="s">
         <v>349</v>
       </c>
@@ -3447,7 +3501,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3">
       <c r="A176" t="s">
         <v>351</v>
       </c>
@@ -3458,7 +3512,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3">
       <c r="A177" t="s">
         <v>353</v>
       </c>
@@ -3469,7 +3523,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3">
       <c r="A178" t="s">
         <v>355</v>
       </c>
@@ -3480,7 +3534,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3">
       <c r="A179" t="s">
         <v>357</v>
       </c>
@@ -3491,7 +3545,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3">
       <c r="A180" t="s">
         <v>359</v>
       </c>
@@ -3502,7 +3556,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3">
       <c r="A181" t="s">
         <v>361</v>
       </c>
@@ -3513,7 +3567,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3">
       <c r="A182" t="s">
         <v>363</v>
       </c>
@@ -3522,6 +3576,105 @@
       </c>
       <c r="C182" t="s">
         <v>270</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3">
+      <c r="A183" t="s">
+        <v>365</v>
+      </c>
+      <c r="B183" t="s">
+        <v>366</v>
+      </c>
+      <c r="C183" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3">
+      <c r="A184" t="s">
+        <v>367</v>
+      </c>
+      <c r="B184" t="s">
+        <v>368</v>
+      </c>
+      <c r="C184" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3">
+      <c r="A185" t="s">
+        <v>369</v>
+      </c>
+      <c r="B185" t="s">
+        <v>370</v>
+      </c>
+      <c r="C185" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3">
+      <c r="A186" t="s">
+        <v>371</v>
+      </c>
+      <c r="B186" t="s">
+        <v>372</v>
+      </c>
+      <c r="C186" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3">
+      <c r="A187" t="s">
+        <v>373</v>
+      </c>
+      <c r="B187" t="s">
+        <v>374</v>
+      </c>
+      <c r="C187" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
+      <c r="A188" t="s">
+        <v>375</v>
+      </c>
+      <c r="B188" t="s">
+        <v>376</v>
+      </c>
+      <c r="C188" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3">
+      <c r="A189" t="s">
+        <v>377</v>
+      </c>
+      <c r="B189" t="s">
+        <v>378</v>
+      </c>
+      <c r="C189" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3">
+      <c r="A190" t="s">
+        <v>379</v>
+      </c>
+      <c r="B190" t="s">
+        <v>380</v>
+      </c>
+      <c r="C190" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3">
+      <c r="A191" t="s">
+        <v>381</v>
+      </c>
+      <c r="B191" t="s">
+        <v>382</v>
+      </c>
+      <c r="C191" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added more jobs 5 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="130" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D751C798-9842-41FC-9857-15A61752D38E}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1CF938-9A9A-4C3F-BD57-B7419AD8CF58}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="395">
   <si>
     <t>Job</t>
   </si>
@@ -1188,6 +1188,42 @@
   </si>
   <si>
     <t>49 Wards Line, Greytown</t>
+  </si>
+  <si>
+    <t>1085554 - 00062941 - DG Label</t>
+  </si>
+  <si>
+    <t>4 Boydfield Street, Whanganui East</t>
+  </si>
+  <si>
+    <t>1085553 - 00057633 - DG Label</t>
+  </si>
+  <si>
+    <t>2a Buxton Road, Westmere</t>
+  </si>
+  <si>
+    <t>1085551 - 00062161 - DG Label</t>
+  </si>
+  <si>
+    <t>72 Watt Street, Featherston</t>
+  </si>
+  <si>
+    <t>1085550 - 00061611 - DG Label</t>
+  </si>
+  <si>
+    <t>180A Manchester Street, Feilding</t>
+  </si>
+  <si>
+    <t>1085549 - 00061578 - DG Label</t>
+  </si>
+  <si>
+    <t>9 Rothesay Place, Highbury</t>
+  </si>
+  <si>
+    <t>1085548 - 00061326 - DG Label</t>
+  </si>
+  <si>
+    <t>19 Mill Grove, Clareville</t>
   </si>
 </sst>
 </file>
@@ -1568,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C191"/>
+  <dimension ref="A1:C197"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -3677,6 +3713,72 @@
         <v>269</v>
       </c>
     </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
+        <v>383</v>
+      </c>
+      <c r="B192" t="s">
+        <v>384</v>
+      </c>
+      <c r="C192" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3">
+      <c r="A193" t="s">
+        <v>385</v>
+      </c>
+      <c r="B193" t="s">
+        <v>386</v>
+      </c>
+      <c r="C193" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3">
+      <c r="A194" t="s">
+        <v>387</v>
+      </c>
+      <c r="B194" t="s">
+        <v>388</v>
+      </c>
+      <c r="C194" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3">
+      <c r="A195" t="s">
+        <v>389</v>
+      </c>
+      <c r="B195" t="s">
+        <v>390</v>
+      </c>
+      <c r="C195" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3">
+      <c r="A196" t="s">
+        <v>391</v>
+      </c>
+      <c r="B196" t="s">
+        <v>392</v>
+      </c>
+      <c r="C196" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
+        <v>393</v>
+      </c>
+      <c r="B197" t="s">
+        <v>394</v>
+      </c>
+      <c r="C197" t="s">
+        <v>270</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added jobs 7 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1CF938-9A9A-4C3F-BD57-B7419AD8CF58}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BB98B0D-F34D-42AF-9F55-7DD09F91BF47}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="415">
   <si>
     <t>Job</t>
   </si>
@@ -1224,13 +1224,73 @@
   </si>
   <si>
     <t>19 Mill Grove, Clareville</t>
+  </si>
+  <si>
+    <t>1085628 - 00042760 - DG Label</t>
+  </si>
+  <si>
+    <t>286 Central Mangaone Road, Eketahuna</t>
+  </si>
+  <si>
+    <t>1085627 - 00060729 - DG Label</t>
+  </si>
+  <si>
+    <t>1294 Turakina Valley Road, Turakina</t>
+  </si>
+  <si>
+    <t>1085626 - 00058779 - DG Label</t>
+  </si>
+  <si>
+    <t>154 Watershed Road, Bunnythorpe</t>
+  </si>
+  <si>
+    <t>1085625 - 00059698 - DG Label</t>
+  </si>
+  <si>
+    <t>19 Bengston Street, Eketahuna</t>
+  </si>
+  <si>
+    <t>1085624 - 00045886 - DG Label</t>
+  </si>
+  <si>
+    <t>17 Pickwick Road, Otamatea</t>
+  </si>
+  <si>
+    <t>1085623 - 00035552 - DG Label</t>
+  </si>
+  <si>
+    <t>15 Tangimoana Road, Ohakea</t>
+  </si>
+  <si>
+    <t>1085622 - 00055340 - DG Label</t>
+  </si>
+  <si>
+    <t>41 Tayforth Road, Whanganui</t>
+  </si>
+  <si>
+    <t>1085621 - 00052867 - DG Label</t>
+  </si>
+  <si>
+    <t>8 Aotea Street, Feilding</t>
+  </si>
+  <si>
+    <t>1085620 - 00053518 - DG Label</t>
+  </si>
+  <si>
+    <t>295 Dalefield Road, Dalefield</t>
+  </si>
+  <si>
+    <t>1085619 - 00054760 - DG Label</t>
+  </si>
+  <si>
+    <t>42 Johnstone Drive, Fitzherbert</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1604,15 +1664,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C197"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:C207"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="64.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1623,7 +1683,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>211</v>
       </c>
@@ -1634,7 +1694,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>213</v>
       </c>
@@ -1645,7 +1705,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>215</v>
       </c>
@@ -1656,7 +1716,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>217</v>
       </c>
@@ -1667,7 +1727,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>219</v>
       </c>
@@ -1678,7 +1738,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>221</v>
       </c>
@@ -1689,7 +1749,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>223</v>
       </c>
@@ -1700,7 +1760,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>225</v>
       </c>
@@ -1711,7 +1771,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>227</v>
       </c>
@@ -1722,7 +1782,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>229</v>
       </c>
@@ -1733,7 +1793,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>231</v>
       </c>
@@ -1744,7 +1804,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>233</v>
       </c>
@@ -1755,7 +1815,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>235</v>
       </c>
@@ -1766,7 +1826,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>237</v>
       </c>
@@ -1777,7 +1837,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>239</v>
       </c>
@@ -1788,7 +1848,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>241</v>
       </c>
@@ -1799,7 +1859,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>243</v>
       </c>
@@ -1810,7 +1870,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>245</v>
       </c>
@@ -1821,7 +1881,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>247</v>
       </c>
@@ -1832,7 +1892,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>249</v>
       </c>
@@ -1843,7 +1903,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>251</v>
       </c>
@@ -1854,7 +1914,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>253</v>
       </c>
@@ -1865,7 +1925,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>255</v>
       </c>
@@ -1876,7 +1936,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>257</v>
       </c>
@@ -1887,7 +1947,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>259</v>
       </c>
@@ -1898,7 +1958,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>260</v>
       </c>
@@ -1909,7 +1969,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>262</v>
       </c>
@@ -1920,7 +1980,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>264</v>
       </c>
@@ -1931,7 +1991,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>266</v>
       </c>
@@ -1942,7 +2002,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>268</v>
       </c>
@@ -1953,7 +2013,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>146</v>
       </c>
@@ -1964,7 +2024,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>147</v>
       </c>
@@ -1975,7 +2035,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>149</v>
       </c>
@@ -1986,7 +2046,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>151</v>
       </c>
@@ -1997,7 +2057,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>153</v>
       </c>
@@ -2008,7 +2068,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>155</v>
       </c>
@@ -2019,7 +2079,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>157</v>
       </c>
@@ -2030,7 +2090,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>159</v>
       </c>
@@ -2041,7 +2101,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>161</v>
       </c>
@@ -2052,7 +2112,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>163</v>
       </c>
@@ -2063,7 +2123,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>165</v>
       </c>
@@ -2074,7 +2134,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>167</v>
       </c>
@@ -2085,7 +2145,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>169</v>
       </c>
@@ -2096,7 +2156,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>171</v>
       </c>
@@ -2107,7 +2167,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>173</v>
       </c>
@@ -2118,7 +2178,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>174</v>
       </c>
@@ -2129,7 +2189,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>176</v>
       </c>
@@ -2140,7 +2200,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>178</v>
       </c>
@@ -2151,7 +2211,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>180</v>
       </c>
@@ -2162,7 +2222,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>181</v>
       </c>
@@ -2173,7 +2233,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>183</v>
       </c>
@@ -2184,7 +2244,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>185</v>
       </c>
@@ -2195,7 +2255,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>187</v>
       </c>
@@ -2206,7 +2266,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>189</v>
       </c>
@@ -2217,7 +2277,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>191</v>
       </c>
@@ -2228,7 +2288,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>193</v>
       </c>
@@ -2239,7 +2299,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>195</v>
       </c>
@@ -2250,7 +2310,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>197</v>
       </c>
@@ -2261,7 +2321,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>199</v>
       </c>
@@ -2272,7 +2332,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>201</v>
       </c>
@@ -2283,7 +2343,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>203</v>
       </c>
@@ -2294,7 +2354,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>205</v>
       </c>
@@ -2305,7 +2365,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>207</v>
       </c>
@@ -2316,7 +2376,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>209</v>
       </c>
@@ -2327,7 +2387,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2338,7 +2398,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -2349,7 +2409,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>5</v>
       </c>
@@ -2360,7 +2420,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>6</v>
       </c>
@@ -2371,7 +2431,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>7</v>
       </c>
@@ -2382,7 +2442,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>8</v>
       </c>
@@ -2393,7 +2453,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>9</v>
       </c>
@@ -2404,7 +2464,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2415,7 +2475,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>13</v>
       </c>
@@ -2426,7 +2486,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>14</v>
       </c>
@@ -2437,7 +2497,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -2448,7 +2508,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>17</v>
       </c>
@@ -2459,7 +2519,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>18</v>
       </c>
@@ -2470,7 +2530,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>19</v>
       </c>
@@ -2481,7 +2541,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>20</v>
       </c>
@@ -2492,7 +2552,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>22</v>
       </c>
@@ -2503,7 +2563,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>24</v>
       </c>
@@ -2514,7 +2574,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>25</v>
       </c>
@@ -2525,7 +2585,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>65</v>
       </c>
@@ -2536,7 +2596,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -2547,7 +2607,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>29</v>
       </c>
@@ -2558,7 +2618,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>31</v>
       </c>
@@ -2569,7 +2629,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>33</v>
       </c>
@@ -2580,7 +2640,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>35</v>
       </c>
@@ -2591,7 +2651,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>37</v>
       </c>
@@ -2602,7 +2662,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>39</v>
       </c>
@@ -2613,7 +2673,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>41</v>
       </c>
@@ -2624,7 +2684,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>43</v>
       </c>
@@ -2635,7 +2695,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>45</v>
       </c>
@@ -2646,7 +2706,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>47</v>
       </c>
@@ -2657,7 +2717,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>49</v>
       </c>
@@ -2668,7 +2728,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>51</v>
       </c>
@@ -2679,7 +2739,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>53</v>
       </c>
@@ -2690,7 +2750,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>55</v>
       </c>
@@ -2701,7 +2761,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>57</v>
       </c>
@@ -2712,7 +2772,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>59</v>
       </c>
@@ -2723,7 +2783,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>61</v>
       </c>
@@ -2734,7 +2794,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>63</v>
       </c>
@@ -2745,7 +2805,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>26</v>
       </c>
@@ -2756,7 +2816,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>67</v>
       </c>
@@ -2767,7 +2827,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>69</v>
       </c>
@@ -2778,7 +2838,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>71</v>
       </c>
@@ -2789,7 +2849,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>73</v>
       </c>
@@ -2800,7 +2860,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>75</v>
       </c>
@@ -2811,7 +2871,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>77</v>
       </c>
@@ -2822,7 +2882,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>79</v>
       </c>
@@ -2833,7 +2893,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>81</v>
       </c>
@@ -2844,7 +2904,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>83</v>
       </c>
@@ -2855,7 +2915,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>84</v>
       </c>
@@ -2866,7 +2926,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>85</v>
       </c>
@@ -2877,7 +2937,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>87</v>
       </c>
@@ -2888,7 +2948,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>89</v>
       </c>
@@ -2899,7 +2959,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>91</v>
       </c>
@@ -2910,7 +2970,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>93</v>
       </c>
@@ -2921,7 +2981,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>95</v>
       </c>
@@ -2932,7 +2992,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>97</v>
       </c>
@@ -2943,7 +3003,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>99</v>
       </c>
@@ -2954,7 +3014,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>101</v>
       </c>
@@ -2965,7 +3025,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>103</v>
       </c>
@@ -2976,7 +3036,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>105</v>
       </c>
@@ -2987,7 +3047,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>107</v>
       </c>
@@ -2998,7 +3058,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>109</v>
       </c>
@@ -3009,7 +3069,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>111</v>
       </c>
@@ -3020,7 +3080,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>113</v>
       </c>
@@ -3031,7 +3091,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>115</v>
       </c>
@@ -3042,7 +3102,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>117</v>
       </c>
@@ -3053,7 +3113,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>119</v>
       </c>
@@ -3064,7 +3124,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>121</v>
       </c>
@@ -3075,7 +3135,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>123</v>
       </c>
@@ -3086,7 +3146,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>125</v>
       </c>
@@ -3097,7 +3157,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>127</v>
       </c>
@@ -3108,7 +3168,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>128</v>
       </c>
@@ -3119,7 +3179,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>130</v>
       </c>
@@ -3130,7 +3190,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>132</v>
       </c>
@@ -3141,7 +3201,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>134</v>
       </c>
@@ -3152,7 +3212,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>136</v>
       </c>
@@ -3163,7 +3223,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>138</v>
       </c>
@@ -3174,7 +3234,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>140</v>
       </c>
@@ -3185,7 +3245,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>142</v>
       </c>
@@ -3196,7 +3256,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="145" spans="1:3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>144</v>
       </c>
@@ -3207,7 +3267,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="146" spans="1:3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>306</v>
       </c>
@@ -3218,7 +3278,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="147" spans="1:3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>305</v>
       </c>
@@ -3229,7 +3289,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>303</v>
       </c>
@@ -3240,7 +3300,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="149" spans="1:3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>301</v>
       </c>
@@ -3251,7 +3311,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>299</v>
       </c>
@@ -3262,7 +3322,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="151" spans="1:3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>297</v>
       </c>
@@ -3273,7 +3333,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="152" spans="1:3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>295</v>
       </c>
@@ -3284,7 +3344,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="153" spans="1:3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>293</v>
       </c>
@@ -3295,7 +3355,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>320</v>
       </c>
@@ -3306,7 +3366,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="155" spans="1:3">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>318</v>
       </c>
@@ -3317,7 +3377,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="156" spans="1:3">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>316</v>
       </c>
@@ -3328,7 +3388,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>314</v>
       </c>
@@ -3339,7 +3399,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="158" spans="1:3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>312</v>
       </c>
@@ -3350,7 +3410,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="159" spans="1:3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>310</v>
       </c>
@@ -3361,7 +3421,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>308</v>
       </c>
@@ -3372,7 +3432,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="161" spans="1:3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>344</v>
       </c>
@@ -3383,7 +3443,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>342</v>
       </c>
@@ -3394,7 +3454,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>340</v>
       </c>
@@ -3405,7 +3465,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>338</v>
       </c>
@@ -3416,7 +3476,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>336</v>
       </c>
@@ -3427,7 +3487,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>334</v>
       </c>
@@ -3438,7 +3498,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>332</v>
       </c>
@@ -3449,7 +3509,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>330</v>
       </c>
@@ -3460,7 +3520,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>328</v>
       </c>
@@ -3471,7 +3531,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="170" spans="1:3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>326</v>
       </c>
@@ -3482,7 +3542,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>324</v>
       </c>
@@ -3493,7 +3553,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>322</v>
       </c>
@@ -3504,7 +3564,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>345</v>
       </c>
@@ -3515,7 +3575,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>347</v>
       </c>
@@ -3526,7 +3586,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>349</v>
       </c>
@@ -3537,7 +3597,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>351</v>
       </c>
@@ -3548,7 +3608,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>353</v>
       </c>
@@ -3559,7 +3619,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>355</v>
       </c>
@@ -3570,7 +3630,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>357</v>
       </c>
@@ -3581,7 +3641,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>359</v>
       </c>
@@ -3592,7 +3652,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>361</v>
       </c>
@@ -3603,7 +3663,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>363</v>
       </c>
@@ -3614,7 +3674,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>365</v>
       </c>
@@ -3625,7 +3685,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>367</v>
       </c>
@@ -3636,7 +3696,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>369</v>
       </c>
@@ -3647,7 +3707,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>371</v>
       </c>
@@ -3658,7 +3718,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>373</v>
       </c>
@@ -3669,7 +3729,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>375</v>
       </c>
@@ -3680,7 +3740,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="189" spans="1:3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>377</v>
       </c>
@@ -3691,7 +3751,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>379</v>
       </c>
@@ -3702,7 +3762,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>381</v>
       </c>
@@ -3713,7 +3773,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>383</v>
       </c>
@@ -3724,7 +3784,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>385</v>
       </c>
@@ -3735,7 +3795,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>387</v>
       </c>
@@ -3746,7 +3806,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>389</v>
       </c>
@@ -3757,7 +3817,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>391</v>
       </c>
@@ -3768,7 +3828,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>393</v>
       </c>
@@ -3776,6 +3836,116 @@
         <v>394</v>
       </c>
       <c r="C197" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>395</v>
+      </c>
+      <c r="B198" t="s">
+        <v>396</v>
+      </c>
+      <c r="C198" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>397</v>
+      </c>
+      <c r="B199" t="s">
+        <v>398</v>
+      </c>
+      <c r="C199" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>399</v>
+      </c>
+      <c r="B200" t="s">
+        <v>400</v>
+      </c>
+      <c r="C200" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>401</v>
+      </c>
+      <c r="B201" t="s">
+        <v>402</v>
+      </c>
+      <c r="C201" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>403</v>
+      </c>
+      <c r="B202" t="s">
+        <v>404</v>
+      </c>
+      <c r="C202" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>405</v>
+      </c>
+      <c r="B203" t="s">
+        <v>406</v>
+      </c>
+      <c r="C203" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>407</v>
+      </c>
+      <c r="B204" t="s">
+        <v>408</v>
+      </c>
+      <c r="C204" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>409</v>
+      </c>
+      <c r="B205" t="s">
+        <v>410</v>
+      </c>
+      <c r="C205" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>411</v>
+      </c>
+      <c r="B206" t="s">
+        <v>412</v>
+      </c>
+      <c r="C206" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>413</v>
+      </c>
+      <c r="B207" t="s">
+        <v>414</v>
+      </c>
+      <c r="C207" t="s">
         <v>270</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added/removed jobs 10 Aug
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BB98B0D-F34D-42AF-9F55-7DD09F91BF47}"/>
+  <xr:revisionPtr revIDLastSave="174" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DF68EE7-DA39-4A83-9138-C38E883080C4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="449">
   <si>
     <t>Job</t>
   </si>
@@ -974,24 +974,6 @@
     <t>1084772 - 00060405 - DG Label</t>
   </si>
   <si>
-    <t>9A Belvedere Crescent, Takaro</t>
-  </si>
-  <si>
-    <t>1084774 - 00053598 - DG Label</t>
-  </si>
-  <si>
-    <t>7 Long Melford Road, Awapuni</t>
-  </si>
-  <si>
-    <t>1084776 - 00045583 - DG Label</t>
-  </si>
-  <si>
-    <t>115 Atawhai Road, Fitzherbert</t>
-  </si>
-  <si>
-    <t>1084778 - 00045588 - DG Label</t>
-  </si>
-  <si>
     <t>74 Cambridge Avenue, Ashhurst</t>
   </si>
   <si>
@@ -1046,12 +1028,6 @@
     <t>1085285 - 00054784 - DG Label</t>
   </si>
   <si>
-    <t>40 Ruapehu Drive, Fitzherbert</t>
-  </si>
-  <si>
-    <t>1085286 - 00056531 - DG Label</t>
-  </si>
-  <si>
     <t>5B Blennerville Close, Marton</t>
   </si>
   <si>
@@ -1284,6 +1260,132 @@
   </si>
   <si>
     <t>42 Johnstone Drive, Fitzherbert</t>
+  </si>
+  <si>
+    <t>1085737 - 00064071 - DG Label</t>
+  </si>
+  <si>
+    <t>471 Lees Road, Feilding</t>
+  </si>
+  <si>
+    <t>1085735 - 00061413 - DG Label</t>
+  </si>
+  <si>
+    <t>85 Watt Street, Featherston</t>
+  </si>
+  <si>
+    <t>1085734 - 00025403 - DG Label</t>
+  </si>
+  <si>
+    <t>7B Brassey Road, Saint Johns Hill</t>
+  </si>
+  <si>
+    <t>1085733 - 00031648 - DG Label</t>
+  </si>
+  <si>
+    <t>9 Fox Road, Springvale</t>
+  </si>
+  <si>
+    <t>1085732 - 00030245 - DG Label</t>
+  </si>
+  <si>
+    <t>47 Kowhai Street, Castlecliff</t>
+  </si>
+  <si>
+    <t>1085731 - 00029753 - DG Label</t>
+  </si>
+  <si>
+    <t>119 Pharazyn Street, Feilding</t>
+  </si>
+  <si>
+    <t>1085730 - 00038535 - DG Label</t>
+  </si>
+  <si>
+    <t>25 Waicola Drive, Fitzherbert</t>
+  </si>
+  <si>
+    <t>1085727 - 00046515 - DG Label</t>
+  </si>
+  <si>
+    <t>6 Hayward Street, Featherston</t>
+  </si>
+  <si>
+    <t>1085726 - 00038396 - DG Label</t>
+  </si>
+  <si>
+    <t>182 Kimbolton Road, Feilding</t>
+  </si>
+  <si>
+    <t>1085725 - 00025168 - DG Label</t>
+  </si>
+  <si>
+    <t>388 Ruakokoputuna Road, Martinborough</t>
+  </si>
+  <si>
+    <t>1085724 - 00032739 - DG Label</t>
+  </si>
+  <si>
+    <t>2187 State Highway 3, Sanson</t>
+  </si>
+  <si>
+    <t>1085722 - 00047186 - DG Label</t>
+  </si>
+  <si>
+    <t>36 Cloverlea Road, Westbrook</t>
+  </si>
+  <si>
+    <t>1085721 - 00054363 - DG Label</t>
+  </si>
+  <si>
+    <t>71 Wightman Road, Sanson</t>
+  </si>
+  <si>
+    <t>1085720 - 00051231 - DG Label</t>
+  </si>
+  <si>
+    <t>14 Spelman Court, Ashhurst</t>
+  </si>
+  <si>
+    <t>1085718 - 00025360 - DG Label</t>
+  </si>
+  <si>
+    <t>65 Hartwell Drive, Bunnythorpe</t>
+  </si>
+  <si>
+    <t>1085717 - 00057960 - DG Label</t>
+  </si>
+  <si>
+    <t>32 Harrison Street West, Featherston</t>
+  </si>
+  <si>
+    <t>1085716 - 00055342 - DG Label</t>
+  </si>
+  <si>
+    <t>52 Surrey Road, Springvale</t>
+  </si>
+  <si>
+    <t>1085715 - 00030535 - DG Label</t>
+  </si>
+  <si>
+    <t>2/31 Moore Street, Tawhero</t>
+  </si>
+  <si>
+    <t>1085714 - 00048298 - DG Label</t>
+  </si>
+  <si>
+    <t>6 Monmouth Street, Feilding</t>
+  </si>
+  <si>
+    <t>1085712 - 00055446 - DG Label</t>
+  </si>
+  <si>
+    <t>262 Campbell Road, Brunswick</t>
+  </si>
+  <si>
+    <t>1085711 - 00060489 - DG Label</t>
+  </si>
+  <si>
+    <t>5 Te Arakura Road, Newbury</t>
   </si>
 </sst>
 </file>
@@ -1664,7 +1766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6218D334-F914-43C7-B5ED-119730E8C2C7}">
-  <dimension ref="A1:C207"/>
+  <dimension ref="A1:C224"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -3357,10 +3459,10 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B154" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="C154" t="s">
         <v>270</v>
@@ -3368,10 +3470,10 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="B155" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C155" t="s">
         <v>269</v>
@@ -3379,21 +3481,21 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B156" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="C156" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="B157" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C157" t="s">
         <v>270</v>
@@ -3401,10 +3503,10 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>312</v>
+        <v>336</v>
       </c>
       <c r="B158" t="s">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="C158" t="s">
         <v>270</v>
@@ -3412,21 +3514,21 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>310</v>
+        <v>334</v>
       </c>
       <c r="B159" t="s">
-        <v>309</v>
+        <v>333</v>
       </c>
       <c r="C159" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>308</v>
+        <v>332</v>
       </c>
       <c r="B160" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
       <c r="C160" t="s">
         <v>270</v>
@@ -3434,10 +3536,10 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="B161" t="s">
-        <v>343</v>
+        <v>329</v>
       </c>
       <c r="C161" t="s">
         <v>270</v>
@@ -3445,21 +3547,21 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="B162" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="C162" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
       <c r="B163" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="C163" t="s">
         <v>270</v>
@@ -3467,21 +3569,21 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>338</v>
+        <v>324</v>
       </c>
       <c r="B164" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="C164" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="B165" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
       <c r="C165" t="s">
         <v>269</v>
@@ -3489,21 +3591,21 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
       <c r="B166" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="C166" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="B167" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
       <c r="C167" t="s">
         <v>270</v>
@@ -3511,10 +3613,10 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="B168" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="C168" t="s">
         <v>269</v>
@@ -3522,10 +3624,10 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="B169" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="C169" t="s">
         <v>269</v>
@@ -3533,10 +3635,10 @@
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="B170" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="C170" t="s">
         <v>270</v>
@@ -3544,10 +3646,10 @@
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="B171" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="C171" t="s">
         <v>270</v>
@@ -3555,10 +3657,10 @@
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
       <c r="B172" t="s">
-        <v>321</v>
+        <v>344</v>
       </c>
       <c r="C172" t="s">
         <v>269</v>
@@ -3572,7 +3674,7 @@
         <v>346</v>
       </c>
       <c r="C173" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
@@ -3583,7 +3685,7 @@
         <v>348</v>
       </c>
       <c r="C174" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
@@ -3594,7 +3696,7 @@
         <v>350</v>
       </c>
       <c r="C175" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
@@ -3605,7 +3707,7 @@
         <v>352</v>
       </c>
       <c r="C176" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
@@ -3616,7 +3718,7 @@
         <v>354</v>
       </c>
       <c r="C177" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
@@ -3627,7 +3729,7 @@
         <v>356</v>
       </c>
       <c r="C178" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
@@ -3649,7 +3751,7 @@
         <v>360</v>
       </c>
       <c r="C180" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -3660,7 +3762,7 @@
         <v>362</v>
       </c>
       <c r="C181" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
@@ -3671,7 +3773,7 @@
         <v>364</v>
       </c>
       <c r="C182" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -3770,7 +3872,7 @@
         <v>382</v>
       </c>
       <c r="C191" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
@@ -3781,7 +3883,7 @@
         <v>384</v>
       </c>
       <c r="C192" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
@@ -3814,7 +3916,7 @@
         <v>390</v>
       </c>
       <c r="C195" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
@@ -3825,7 +3927,7 @@
         <v>392</v>
       </c>
       <c r="C196" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
@@ -3847,7 +3949,7 @@
         <v>396</v>
       </c>
       <c r="C198" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
@@ -3891,7 +3993,7 @@
         <v>404</v>
       </c>
       <c r="C202" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
@@ -3902,7 +4004,7 @@
         <v>406</v>
       </c>
       <c r="C203" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
@@ -3913,7 +4015,7 @@
         <v>408</v>
       </c>
       <c r="C204" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
@@ -3924,7 +4026,7 @@
         <v>410</v>
       </c>
       <c r="C205" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
@@ -3947,6 +4049,193 @@
       </c>
       <c r="C207" t="s">
         <v>270</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>415</v>
+      </c>
+      <c r="B208" t="s">
+        <v>416</v>
+      </c>
+      <c r="C208" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>417</v>
+      </c>
+      <c r="B209" t="s">
+        <v>418</v>
+      </c>
+      <c r="C209" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>419</v>
+      </c>
+      <c r="B210" t="s">
+        <v>420</v>
+      </c>
+      <c r="C210" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>421</v>
+      </c>
+      <c r="B211" t="s">
+        <v>422</v>
+      </c>
+      <c r="C211" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>423</v>
+      </c>
+      <c r="B212" t="s">
+        <v>424</v>
+      </c>
+      <c r="C212" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>425</v>
+      </c>
+      <c r="B213" t="s">
+        <v>426</v>
+      </c>
+      <c r="C213" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>427</v>
+      </c>
+      <c r="B214" t="s">
+        <v>428</v>
+      </c>
+      <c r="C214" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>429</v>
+      </c>
+      <c r="B215" t="s">
+        <v>430</v>
+      </c>
+      <c r="C215" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>431</v>
+      </c>
+      <c r="B216" t="s">
+        <v>432</v>
+      </c>
+      <c r="C216" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>433</v>
+      </c>
+      <c r="B217" t="s">
+        <v>434</v>
+      </c>
+      <c r="C217" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>435</v>
+      </c>
+      <c r="B218" t="s">
+        <v>436</v>
+      </c>
+      <c r="C218" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>437</v>
+      </c>
+      <c r="B219" t="s">
+        <v>438</v>
+      </c>
+      <c r="C219" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>439</v>
+      </c>
+      <c r="B220" t="s">
+        <v>440</v>
+      </c>
+      <c r="C220" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>441</v>
+      </c>
+      <c r="B221" t="s">
+        <v>442</v>
+      </c>
+      <c r="C221" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>443</v>
+      </c>
+      <c r="B222" t="s">
+        <v>444</v>
+      </c>
+      <c r="C222" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>445</v>
+      </c>
+      <c r="B223" t="s">
+        <v>446</v>
+      </c>
+      <c r="C223" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>447</v>
+      </c>
+      <c r="B224" t="s">
+        <v>448</v>
+      </c>
+      <c r="C224" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish spreadsheet update via web page
</commit_message>
<xml_diff>
--- a/DGS LIST.xlsx
+++ b/DGS LIST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://feisst-my.sharepoint.com/personal/chisora_h_npe-tech_co_nz/Documents/Documents/DG-Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="174" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3DF68EE7-DA39-4A83-9138-C38E883080C4}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="8_{CCCF0366-673B-4613-8CFF-E13952FC8332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37618238-51C5-49B9-9327-84E12C9B4DA4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-330" windowWidth="29040" windowHeight="15720" xr2:uid="{F977427A-6EEF-496F-83AC-E1A3F4E254D6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="393">
   <si>
     <t>Job</t>
   </si>
@@ -674,171 +674,6 @@
     <t>34 Jellicoe Street, Martinborough</t>
   </si>
   <si>
-    <t>1082613 - 00037301  - DG Label - 0068841000WR999</t>
-  </si>
-  <si>
-    <t>663 CHESTER ROAD , WEST TARATAHI, CARTERTON, 5791</t>
-  </si>
-  <si>
-    <t>1082609 - 00037241  - DG Label - 1000572372PC23E</t>
-  </si>
-  <si>
-    <t>11 Te Ore Ore Bideford Road , Te Ore Ore, Masterton, 5886</t>
-  </si>
-  <si>
-    <t>1082608 - 00037238  - DG Label - 1000605901PC3C4</t>
-  </si>
-  <si>
-    <t>32 TAMA ROAD , RIVERSDALE BEACH, MASTERTON, 5872</t>
-  </si>
-  <si>
-    <t>1082604 - 00037235 - DG Label - 1000583813PC6B9</t>
-  </si>
-  <si>
-    <t>39A WELD STREET , MARTINBOROUGH, MARTINBOROUGH, 5711</t>
-  </si>
-  <si>
-    <t>1082601 - 00036842 - DG Label - 1000544375PCB18</t>
-  </si>
-  <si>
-    <t>9 FAIRWAY DR , MARTINBOROUGH, MARTINBOROUGH, 5784</t>
-  </si>
-  <si>
-    <t>1082588 - 00035665 - DG Label - 1000624084PCAA5</t>
-  </si>
-  <si>
-    <t>219B GLENMORVEN ROAD , MORISON BUSH, GREYTOWN, 5794</t>
-  </si>
-  <si>
-    <t>1082586 - 00035670 - DG Label - 0060007400WR56A</t>
-  </si>
-  <si>
-    <t>274 HIGH STREET NORTH , CARTERTON, 5713</t>
-  </si>
-  <si>
-    <t>1082585 - 00035668 - DG Label - 0666003845PCD5A</t>
-  </si>
-  <si>
-    <t>433B WAIOHINE GORGE ROAD , CARTERTON, 5791</t>
-  </si>
-  <si>
-    <t>1082584 - 00034018 - DG Label - 0052489000WRDDE</t>
-  </si>
-  <si>
-    <t>1 TAMARISK DR , MASTERTON</t>
-  </si>
-  <si>
-    <t>1082582 - 00034014  - DG Label -0070568100WR40F</t>
-  </si>
-  <si>
-    <t>17 HOMESTEAD LANE , GREYTOWN, GREYTOWN, 5712</t>
-  </si>
-  <si>
-    <t>1082576 - 00031683  - DG Label -0666003622PC96B</t>
-  </si>
-  <si>
-    <t>70B DUBLIN STREET , MARTINBOROUGH, 5711</t>
-  </si>
-  <si>
-    <t>1082574 - 00014488  - DG Label -0037559000WRE8B</t>
-  </si>
-  <si>
-    <t>64 CORNWALL STREET , MASTERTON, 5810</t>
-  </si>
-  <si>
-    <t>1082571 - 00039316 - DG Label - 0000068226CP3F0</t>
-  </si>
-  <si>
-    <t>2 VISCOUNT PLACE, WEST END, PALMERSTON NORTH, 4412</t>
-  </si>
-  <si>
-    <t>1082562 - 00052452 - DG Label - 0000080600CP356</t>
-  </si>
-  <si>
-    <t>69 KERERU DRIVE, TURITEA, PALMERSTON NORTH, 4472</t>
-  </si>
-  <si>
-    <t>1082560 - 00052590 - DG Label - 0000048858CP6F1</t>
-  </si>
-  <si>
-    <t>9 HEATHCOTE PLACE, FITZHERBERT, PALMERSTON NORTH, 4410</t>
-  </si>
-  <si>
-    <t>1082527 - 00052277 - DG Label - 0000065056CP68A</t>
-  </si>
-  <si>
-    <t>180B PHARAZYN ROAD, FEILDING, 4777</t>
-  </si>
-  <si>
-    <t>1082526 - 00044306 - DG Label - 1000605858PCC99</t>
-  </si>
-  <si>
-    <t>1 Cotterville Crescent, Greytown, 5712</t>
-  </si>
-  <si>
-    <t>1082525 - 00042914 - DG Label - 1000574372PC7FE</t>
-  </si>
-  <si>
-    <t>13 MERVYN BROWN PLACE, SOLWAY, MASTERTON, 5810</t>
-  </si>
-  <si>
-    <t>1082504 - 00050338 - DG Label - 1000579124PCE5E</t>
-  </si>
-  <si>
-    <t>4 HUFFINGTON PLACE, FEILDING, FEILDING, 4702</t>
-  </si>
-  <si>
-    <t>1082503 - 00050326 - DG Label - 0900086275PCEC2</t>
-  </si>
-  <si>
-    <t>15 RON PLACE, FITZHERBERT, PALMERSTON NORTH, 4410</t>
-  </si>
-  <si>
-    <t>1082492 - 00055639 - DG Label - 0000037890CP0D3</t>
-  </si>
-  <si>
-    <t>41 ESCORT GROVE, AWAPUNI, PALMERSTON NORTH, 4412</t>
-  </si>
-  <si>
-    <t>1082489 - 00042252 - DG Label - 0666001531PCF45</t>
-  </si>
-  <si>
-    <t>221B State Highway 2, Opaki, Masterton, 5871</t>
-  </si>
-  <si>
-    <t>1082487 - 00042599 - DG Label - 0070237600WR412</t>
-  </si>
-  <si>
-    <t>16 PAPAWAI ROAD, GREYTOWN</t>
-  </si>
-  <si>
-    <t>1082485 - 00052302 - DG Label - 1000615865PCCDB</t>
-  </si>
-  <si>
-    <t>8 GRATITUDE WAY, KELVIN GROVE, PALMERSTON NORTH, 4470</t>
-  </si>
-  <si>
-    <t>1082477 - 00052899 - DG Label- 1000594314PC4FC</t>
-  </si>
-  <si>
-    <t>1082458 - 00054943 - DG Label - 1000624687PC063</t>
-  </si>
-  <si>
-    <t>8 Sardinia Grove, Fitzherbert, Palmerston North</t>
-  </si>
-  <si>
-    <t>1082455 - 00044025 - DG Label - 1000621883PC042</t>
-  </si>
-  <si>
-    <t>6 CASTLEBRIDGE LANE, AOKAUTERE, PALMERSTON NORTH, 4471</t>
-  </si>
-  <si>
-    <t>1082446 - 00050624 - DG Label - 1000580901PC775</t>
-  </si>
-  <si>
-    <t>43 COUTTS WAY, FITZHERBERT, PALMERSTON NORTH, 4410</t>
-  </si>
-  <si>
     <t>1077616 - 00029329  - DG Label</t>
   </si>
   <si>
@@ -912,9 +747,6 @@
   </si>
   <si>
     <t>688 Aranui Road, Kairanga</t>
-  </si>
-  <si>
-    <t>26 MAKOPUA ROAD, TAOROA JUNCTION</t>
   </si>
   <si>
     <t>45D Brandon Street, Featherston</t>
@@ -1782,337 +1614,29 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B2" t="s">
-        <v>212</v>
-      </c>
-      <c r="C2" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B3" t="s">
-        <v>214</v>
-      </c>
-      <c r="C3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C4" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
         <v>217</v>
-      </c>
-      <c r="B5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C5" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>219</v>
-      </c>
-      <c r="B6" t="s">
-        <v>220</v>
-      </c>
-      <c r="C6" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>221</v>
-      </c>
-      <c r="B7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C7" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>223</v>
-      </c>
-      <c r="B8" t="s">
-        <v>224</v>
-      </c>
-      <c r="C8" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>225</v>
-      </c>
-      <c r="B9" t="s">
-        <v>226</v>
-      </c>
-      <c r="C9" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>227</v>
-      </c>
-      <c r="B10" t="s">
-        <v>228</v>
-      </c>
-      <c r="C10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>229</v>
-      </c>
-      <c r="B11" t="s">
-        <v>230</v>
-      </c>
-      <c r="C11" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>231</v>
-      </c>
-      <c r="B12" t="s">
-        <v>232</v>
-      </c>
-      <c r="C12" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>233</v>
-      </c>
-      <c r="B13" t="s">
-        <v>234</v>
-      </c>
-      <c r="C13" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>235</v>
-      </c>
-      <c r="B14" t="s">
-        <v>236</v>
-      </c>
-      <c r="C14" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>237</v>
-      </c>
-      <c r="B15" t="s">
-        <v>238</v>
-      </c>
-      <c r="C15" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>239</v>
-      </c>
-      <c r="B16" t="s">
-        <v>240</v>
-      </c>
-      <c r="C16" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>241</v>
-      </c>
-      <c r="B17" t="s">
-        <v>242</v>
-      </c>
-      <c r="C17" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>243</v>
-      </c>
-      <c r="B18" t="s">
-        <v>244</v>
-      </c>
-      <c r="C18" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>245</v>
-      </c>
-      <c r="B19" t="s">
-        <v>246</v>
-      </c>
-      <c r="C19" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>247</v>
-      </c>
-      <c r="B20" t="s">
-        <v>248</v>
-      </c>
-      <c r="C20" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>249</v>
-      </c>
-      <c r="B21" t="s">
-        <v>250</v>
-      </c>
-      <c r="C21" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>251</v>
-      </c>
-      <c r="B22" t="s">
-        <v>252</v>
-      </c>
-      <c r="C22" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>253</v>
-      </c>
-      <c r="B23" t="s">
-        <v>254</v>
-      </c>
-      <c r="C23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>255</v>
-      </c>
-      <c r="B24" t="s">
-        <v>256</v>
-      </c>
-      <c r="C24" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>257</v>
-      </c>
-      <c r="B25" t="s">
-        <v>258</v>
-      </c>
-      <c r="C25" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>259</v>
-      </c>
-      <c r="B26" t="s">
-        <v>291</v>
-      </c>
-      <c r="C26" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>260</v>
-      </c>
-      <c r="B27" t="s">
-        <v>261</v>
-      </c>
-      <c r="C27" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>262</v>
-      </c>
-      <c r="B28" t="s">
-        <v>263</v>
-      </c>
-      <c r="C28" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>264</v>
-      </c>
-      <c r="B29" t="s">
-        <v>265</v>
-      </c>
-      <c r="C29" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>266</v>
+        <v>211</v>
       </c>
       <c r="B30" t="s">
-        <v>267</v>
+        <v>212</v>
       </c>
       <c r="C30" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>268</v>
+        <v>213</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>235</v>
       </c>
       <c r="C31" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -2120,10 +1644,10 @@
         <v>146</v>
       </c>
       <c r="B32" t="s">
-        <v>289</v>
+        <v>234</v>
       </c>
       <c r="C32" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2134,7 +1658,7 @@
         <v>148</v>
       </c>
       <c r="C33" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -2145,7 +1669,7 @@
         <v>150</v>
       </c>
       <c r="C34" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -2156,7 +1680,7 @@
         <v>152</v>
       </c>
       <c r="C35" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -2167,7 +1691,7 @@
         <v>154</v>
       </c>
       <c r="C36" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -2178,7 +1702,7 @@
         <v>156</v>
       </c>
       <c r="C37" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -2189,7 +1713,7 @@
         <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -2200,7 +1724,7 @@
         <v>160</v>
       </c>
       <c r="C39" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -2211,7 +1735,7 @@
         <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -2222,7 +1746,7 @@
         <v>164</v>
       </c>
       <c r="C41" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -2233,7 +1757,7 @@
         <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -2244,7 +1768,7 @@
         <v>168</v>
       </c>
       <c r="C43" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -2255,7 +1779,7 @@
         <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -2266,7 +1790,7 @@
         <v>172</v>
       </c>
       <c r="C45" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -2274,10 +1798,10 @@
         <v>173</v>
       </c>
       <c r="B46" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="C46" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -2288,7 +1812,7 @@
         <v>175</v>
       </c>
       <c r="C47" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -2299,7 +1823,7 @@
         <v>177</v>
       </c>
       <c r="C48" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -2310,7 +1834,7 @@
         <v>179</v>
       </c>
       <c r="C49" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -2321,7 +1845,7 @@
         <v>179</v>
       </c>
       <c r="C50" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -2332,7 +1856,7 @@
         <v>182</v>
       </c>
       <c r="C51" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -2343,7 +1867,7 @@
         <v>184</v>
       </c>
       <c r="C52" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -2354,7 +1878,7 @@
         <v>186</v>
       </c>
       <c r="C53" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -2365,7 +1889,7 @@
         <v>188</v>
       </c>
       <c r="C54" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -2376,7 +1900,7 @@
         <v>190</v>
       </c>
       <c r="C55" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -2387,7 +1911,7 @@
         <v>192</v>
       </c>
       <c r="C56" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -2398,7 +1922,7 @@
         <v>194</v>
       </c>
       <c r="C57" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -2409,7 +1933,7 @@
         <v>196</v>
       </c>
       <c r="C58" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -2420,7 +1944,7 @@
         <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -2431,7 +1955,7 @@
         <v>200</v>
       </c>
       <c r="C60" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -2442,7 +1966,7 @@
         <v>202</v>
       </c>
       <c r="C61" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -2453,7 +1977,7 @@
         <v>204</v>
       </c>
       <c r="C62" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -2464,7 +1988,7 @@
         <v>206</v>
       </c>
       <c r="C63" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -2475,7 +1999,7 @@
         <v>208</v>
       </c>
       <c r="C64" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -2486,7 +2010,7 @@
         <v>210</v>
       </c>
       <c r="C65" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -2494,10 +2018,10 @@
         <v>2</v>
       </c>
       <c r="B66" t="s">
-        <v>271</v>
+        <v>216</v>
       </c>
       <c r="C66" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -2508,7 +2032,7 @@
         <v>4</v>
       </c>
       <c r="C67" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -2516,10 +2040,10 @@
         <v>5</v>
       </c>
       <c r="B68" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C68" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -2527,10 +2051,10 @@
         <v>6</v>
       </c>
       <c r="B69" t="s">
-        <v>274</v>
+        <v>219</v>
       </c>
       <c r="C69" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -2538,10 +2062,10 @@
         <v>7</v>
       </c>
       <c r="B70" t="s">
-        <v>275</v>
+        <v>220</v>
       </c>
       <c r="C70" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -2549,10 +2073,10 @@
         <v>8</v>
       </c>
       <c r="B71" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="C71" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -2563,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="C72" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -2574,7 +2098,7 @@
         <v>12</v>
       </c>
       <c r="C73" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -2582,10 +2106,10 @@
         <v>13</v>
       </c>
       <c r="B74" t="s">
-        <v>277</v>
+        <v>222</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -2596,7 +2120,7 @@
         <v>15</v>
       </c>
       <c r="C75" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -2604,10 +2128,10 @@
         <v>16</v>
       </c>
       <c r="B76" t="s">
-        <v>287</v>
+        <v>232</v>
       </c>
       <c r="C76" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -2615,10 +2139,10 @@
         <v>17</v>
       </c>
       <c r="B77" t="s">
-        <v>278</v>
+        <v>223</v>
       </c>
       <c r="C77" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -2626,10 +2150,10 @@
         <v>18</v>
       </c>
       <c r="B78" t="s">
-        <v>279</v>
+        <v>224</v>
       </c>
       <c r="C78" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -2637,10 +2161,10 @@
         <v>19</v>
       </c>
       <c r="B79" t="s">
-        <v>280</v>
+        <v>225</v>
       </c>
       <c r="C79" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -2651,7 +2175,7 @@
         <v>21</v>
       </c>
       <c r="C80" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -2662,7 +2186,7 @@
         <v>23</v>
       </c>
       <c r="C81" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -2670,10 +2194,10 @@
         <v>24</v>
       </c>
       <c r="B82" t="s">
-        <v>285</v>
+        <v>230</v>
       </c>
       <c r="C82" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -2681,10 +2205,10 @@
         <v>25</v>
       </c>
       <c r="B83" t="s">
-        <v>286</v>
+        <v>231</v>
       </c>
       <c r="C83" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -2695,7 +2219,7 @@
         <v>66</v>
       </c>
       <c r="C84" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -2706,7 +2230,7 @@
         <v>28</v>
       </c>
       <c r="C85" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -2717,7 +2241,7 @@
         <v>30</v>
       </c>
       <c r="C86" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -2728,7 +2252,7 @@
         <v>32</v>
       </c>
       <c r="C87" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -2739,7 +2263,7 @@
         <v>34</v>
       </c>
       <c r="C88" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -2750,7 +2274,7 @@
         <v>36</v>
       </c>
       <c r="C89" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -2761,7 +2285,7 @@
         <v>38</v>
       </c>
       <c r="C90" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -2772,7 +2296,7 @@
         <v>40</v>
       </c>
       <c r="C91" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -2783,7 +2307,7 @@
         <v>42</v>
       </c>
       <c r="C92" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -2794,7 +2318,7 @@
         <v>44</v>
       </c>
       <c r="C93" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -2805,7 +2329,7 @@
         <v>46</v>
       </c>
       <c r="C94" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -2816,7 +2340,7 @@
         <v>48</v>
       </c>
       <c r="C95" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -2827,7 +2351,7 @@
         <v>50</v>
       </c>
       <c r="C96" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -2838,7 +2362,7 @@
         <v>52</v>
       </c>
       <c r="C97" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -2849,7 +2373,7 @@
         <v>54</v>
       </c>
       <c r="C98" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -2860,7 +2384,7 @@
         <v>56</v>
       </c>
       <c r="C99" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -2871,7 +2395,7 @@
         <v>58</v>
       </c>
       <c r="C100" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -2882,7 +2406,7 @@
         <v>60</v>
       </c>
       <c r="C101" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -2893,7 +2417,7 @@
         <v>62</v>
       </c>
       <c r="C102" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -2904,7 +2428,7 @@
         <v>64</v>
       </c>
       <c r="C103" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -2912,10 +2436,10 @@
         <v>26</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>281</v>
+        <v>226</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -2926,7 +2450,7 @@
         <v>68</v>
       </c>
       <c r="C105" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -2937,7 +2461,7 @@
         <v>70</v>
       </c>
       <c r="C106" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -2948,7 +2472,7 @@
         <v>72</v>
       </c>
       <c r="C107" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -2959,7 +2483,7 @@
         <v>74</v>
       </c>
       <c r="C108" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -2970,7 +2494,7 @@
         <v>76</v>
       </c>
       <c r="C109" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -2981,7 +2505,7 @@
         <v>78</v>
       </c>
       <c r="C110" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
@@ -2992,7 +2516,7 @@
         <v>80</v>
       </c>
       <c r="C111" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
@@ -3003,7 +2527,7 @@
         <v>82</v>
       </c>
       <c r="C112" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
@@ -3011,10 +2535,10 @@
         <v>83</v>
       </c>
       <c r="B113" t="s">
-        <v>282</v>
+        <v>227</v>
       </c>
       <c r="C113" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
@@ -3022,10 +2546,10 @@
         <v>84</v>
       </c>
       <c r="B114" t="s">
-        <v>284</v>
+        <v>229</v>
       </c>
       <c r="C114" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
@@ -3036,7 +2560,7 @@
         <v>86</v>
       </c>
       <c r="C115" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
@@ -3047,7 +2571,7 @@
         <v>88</v>
       </c>
       <c r="C116" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
@@ -3058,7 +2582,7 @@
         <v>90</v>
       </c>
       <c r="C117" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
@@ -3069,7 +2593,7 @@
         <v>92</v>
       </c>
       <c r="C118" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
@@ -3080,7 +2604,7 @@
         <v>94</v>
       </c>
       <c r="C119" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
@@ -3091,7 +2615,7 @@
         <v>96</v>
       </c>
       <c r="C120" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
@@ -3102,7 +2626,7 @@
         <v>98</v>
       </c>
       <c r="C121" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
@@ -3113,7 +2637,7 @@
         <v>100</v>
       </c>
       <c r="C122" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
@@ -3124,7 +2648,7 @@
         <v>102</v>
       </c>
       <c r="C123" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
@@ -3135,7 +2659,7 @@
         <v>104</v>
       </c>
       <c r="C124" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
@@ -3146,7 +2670,7 @@
         <v>106</v>
       </c>
       <c r="C125" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
@@ -3157,7 +2681,7 @@
         <v>108</v>
       </c>
       <c r="C126" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
@@ -3168,7 +2692,7 @@
         <v>110</v>
       </c>
       <c r="C127" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
@@ -3179,7 +2703,7 @@
         <v>112</v>
       </c>
       <c r="C128" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
@@ -3190,7 +2714,7 @@
         <v>114</v>
       </c>
       <c r="C129" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
@@ -3201,7 +2725,7 @@
         <v>116</v>
       </c>
       <c r="C130" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
@@ -3212,7 +2736,7 @@
         <v>118</v>
       </c>
       <c r="C131" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -3223,7 +2747,7 @@
         <v>120</v>
       </c>
       <c r="C132" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
@@ -3234,7 +2758,7 @@
         <v>122</v>
       </c>
       <c r="C133" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -3245,7 +2769,7 @@
         <v>124</v>
       </c>
       <c r="C134" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
@@ -3256,7 +2780,7 @@
         <v>126</v>
       </c>
       <c r="C135" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
@@ -3264,10 +2788,10 @@
         <v>127</v>
       </c>
       <c r="B136" t="s">
-        <v>283</v>
+        <v>228</v>
       </c>
       <c r="C136" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
@@ -3278,7 +2802,7 @@
         <v>129</v>
       </c>
       <c r="C137" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
@@ -3289,7 +2813,7 @@
         <v>131</v>
       </c>
       <c r="C138" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
@@ -3300,7 +2824,7 @@
         <v>133</v>
       </c>
       <c r="C139" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
@@ -3311,7 +2835,7 @@
         <v>135</v>
       </c>
       <c r="C140" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
@@ -3322,7 +2846,7 @@
         <v>137</v>
       </c>
       <c r="C141" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
@@ -3333,7 +2857,7 @@
         <v>139</v>
       </c>
       <c r="C142" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
@@ -3344,7 +2868,7 @@
         <v>141</v>
       </c>
       <c r="C143" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
@@ -3355,7 +2879,7 @@
         <v>143</v>
       </c>
       <c r="C144" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
@@ -3366,876 +2890,876 @@
         <v>145</v>
       </c>
       <c r="C145" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>306</v>
+        <v>250</v>
       </c>
       <c r="B146" t="s">
         <v>135</v>
       </c>
       <c r="C146" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>305</v>
+        <v>249</v>
       </c>
       <c r="B147" t="s">
-        <v>304</v>
+        <v>248</v>
       </c>
       <c r="C147" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>303</v>
+        <v>247</v>
       </c>
       <c r="B148" t="s">
-        <v>302</v>
+        <v>246</v>
       </c>
       <c r="C148" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>301</v>
+        <v>245</v>
       </c>
       <c r="B149" t="s">
-        <v>300</v>
+        <v>244</v>
       </c>
       <c r="C149" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>299</v>
+        <v>243</v>
       </c>
       <c r="B150" t="s">
-        <v>298</v>
+        <v>242</v>
       </c>
       <c r="C150" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>297</v>
+        <v>241</v>
       </c>
       <c r="B151" t="s">
-        <v>296</v>
+        <v>240</v>
       </c>
       <c r="C151" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>295</v>
+        <v>239</v>
       </c>
       <c r="B152" t="s">
-        <v>294</v>
+        <v>238</v>
       </c>
       <c r="C152" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>293</v>
+        <v>237</v>
       </c>
       <c r="B153" t="s">
-        <v>292</v>
+        <v>236</v>
       </c>
       <c r="C153" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>314</v>
+        <v>258</v>
       </c>
       <c r="B154" t="s">
-        <v>313</v>
+        <v>257</v>
       </c>
       <c r="C154" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>312</v>
+        <v>256</v>
       </c>
       <c r="B155" t="s">
-        <v>311</v>
+        <v>255</v>
       </c>
       <c r="C155" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>310</v>
+        <v>254</v>
       </c>
       <c r="B156" t="s">
-        <v>309</v>
+        <v>253</v>
       </c>
       <c r="C156" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>308</v>
+        <v>252</v>
       </c>
       <c r="B157" t="s">
-        <v>307</v>
+        <v>251</v>
       </c>
       <c r="C157" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>336</v>
+        <v>280</v>
       </c>
       <c r="B158" t="s">
-        <v>335</v>
+        <v>279</v>
       </c>
       <c r="C158" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>334</v>
+        <v>278</v>
       </c>
       <c r="B159" t="s">
-        <v>333</v>
+        <v>277</v>
       </c>
       <c r="C159" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>332</v>
+        <v>276</v>
       </c>
       <c r="B160" t="s">
-        <v>331</v>
+        <v>275</v>
       </c>
       <c r="C160" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>330</v>
+        <v>274</v>
       </c>
       <c r="B161" t="s">
-        <v>329</v>
+        <v>273</v>
       </c>
       <c r="C161" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>328</v>
+        <v>272</v>
       </c>
       <c r="B162" t="s">
-        <v>327</v>
+        <v>271</v>
       </c>
       <c r="C162" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>326</v>
+        <v>270</v>
       </c>
       <c r="B163" t="s">
-        <v>325</v>
+        <v>269</v>
       </c>
       <c r="C163" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>324</v>
+        <v>268</v>
       </c>
       <c r="B164" t="s">
-        <v>323</v>
+        <v>267</v>
       </c>
       <c r="C164" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>322</v>
+        <v>266</v>
       </c>
       <c r="B165" t="s">
-        <v>321</v>
+        <v>265</v>
       </c>
       <c r="C165" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>320</v>
+        <v>264</v>
       </c>
       <c r="B166" t="s">
-        <v>319</v>
+        <v>263</v>
       </c>
       <c r="C166" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>318</v>
+        <v>262</v>
       </c>
       <c r="B167" t="s">
-        <v>317</v>
+        <v>261</v>
       </c>
       <c r="C167" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>316</v>
+        <v>260</v>
       </c>
       <c r="B168" t="s">
-        <v>315</v>
+        <v>259</v>
       </c>
       <c r="C168" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>337</v>
+        <v>281</v>
       </c>
       <c r="B169" t="s">
-        <v>338</v>
+        <v>282</v>
       </c>
       <c r="C169" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>339</v>
+        <v>283</v>
       </c>
       <c r="B170" t="s">
-        <v>340</v>
+        <v>284</v>
       </c>
       <c r="C170" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>341</v>
+        <v>285</v>
       </c>
       <c r="B171" t="s">
-        <v>342</v>
+        <v>286</v>
       </c>
       <c r="C171" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>343</v>
+        <v>287</v>
       </c>
       <c r="B172" t="s">
-        <v>344</v>
+        <v>288</v>
       </c>
       <c r="C172" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>345</v>
+        <v>289</v>
       </c>
       <c r="B173" t="s">
-        <v>346</v>
+        <v>290</v>
       </c>
       <c r="C173" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>347</v>
+        <v>291</v>
       </c>
       <c r="B174" t="s">
-        <v>348</v>
+        <v>292</v>
       </c>
       <c r="C174" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>349</v>
+        <v>293</v>
       </c>
       <c r="B175" t="s">
-        <v>350</v>
+        <v>294</v>
       </c>
       <c r="C175" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>351</v>
+        <v>295</v>
       </c>
       <c r="B176" t="s">
-        <v>352</v>
+        <v>296</v>
       </c>
       <c r="C176" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>353</v>
+        <v>297</v>
       </c>
       <c r="B177" t="s">
-        <v>354</v>
+        <v>298</v>
       </c>
       <c r="C177" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>355</v>
+        <v>299</v>
       </c>
       <c r="B178" t="s">
-        <v>356</v>
+        <v>300</v>
       </c>
       <c r="C178" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>357</v>
+        <v>301</v>
       </c>
       <c r="B179" t="s">
-        <v>358</v>
+        <v>302</v>
       </c>
       <c r="C179" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>359</v>
+        <v>303</v>
       </c>
       <c r="B180" t="s">
-        <v>360</v>
+        <v>304</v>
       </c>
       <c r="C180" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>361</v>
+        <v>305</v>
       </c>
       <c r="B181" t="s">
-        <v>362</v>
+        <v>306</v>
       </c>
       <c r="C181" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>363</v>
+        <v>307</v>
       </c>
       <c r="B182" t="s">
-        <v>364</v>
+        <v>308</v>
       </c>
       <c r="C182" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>365</v>
+        <v>309</v>
       </c>
       <c r="B183" t="s">
-        <v>366</v>
+        <v>310</v>
       </c>
       <c r="C183" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>367</v>
+        <v>311</v>
       </c>
       <c r="B184" t="s">
-        <v>368</v>
+        <v>312</v>
       </c>
       <c r="C184" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>369</v>
+        <v>313</v>
       </c>
       <c r="B185" t="s">
-        <v>370</v>
+        <v>314</v>
       </c>
       <c r="C185" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>371</v>
+        <v>315</v>
       </c>
       <c r="B186" t="s">
-        <v>372</v>
+        <v>316</v>
       </c>
       <c r="C186" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>373</v>
+        <v>317</v>
       </c>
       <c r="B187" t="s">
-        <v>374</v>
+        <v>318</v>
       </c>
       <c r="C187" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>375</v>
+        <v>319</v>
       </c>
       <c r="B188" t="s">
-        <v>376</v>
+        <v>320</v>
       </c>
       <c r="C188" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>377</v>
+        <v>321</v>
       </c>
       <c r="B189" t="s">
-        <v>378</v>
+        <v>322</v>
       </c>
       <c r="C189" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>379</v>
+        <v>323</v>
       </c>
       <c r="B190" t="s">
-        <v>380</v>
+        <v>324</v>
       </c>
       <c r="C190" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>381</v>
+        <v>325</v>
       </c>
       <c r="B191" t="s">
-        <v>382</v>
+        <v>326</v>
       </c>
       <c r="C191" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>383</v>
+        <v>327</v>
       </c>
       <c r="B192" t="s">
-        <v>384</v>
+        <v>328</v>
       </c>
       <c r="C192" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>385</v>
+        <v>329</v>
       </c>
       <c r="B193" t="s">
-        <v>386</v>
+        <v>330</v>
       </c>
       <c r="C193" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>387</v>
+        <v>331</v>
       </c>
       <c r="B194" t="s">
-        <v>388</v>
+        <v>332</v>
       </c>
       <c r="C194" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>389</v>
+        <v>333</v>
       </c>
       <c r="B195" t="s">
-        <v>390</v>
+        <v>334</v>
       </c>
       <c r="C195" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>391</v>
+        <v>335</v>
       </c>
       <c r="B196" t="s">
-        <v>392</v>
+        <v>336</v>
       </c>
       <c r="C196" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>393</v>
+        <v>337</v>
       </c>
       <c r="B197" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="C197" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>395</v>
+        <v>339</v>
       </c>
       <c r="B198" t="s">
-        <v>396</v>
+        <v>340</v>
       </c>
       <c r="C198" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>397</v>
+        <v>341</v>
       </c>
       <c r="B199" t="s">
-        <v>398</v>
+        <v>342</v>
       </c>
       <c r="C199" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>399</v>
+        <v>343</v>
       </c>
       <c r="B200" t="s">
-        <v>400</v>
+        <v>344</v>
       </c>
       <c r="C200" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>401</v>
+        <v>345</v>
       </c>
       <c r="B201" t="s">
-        <v>402</v>
+        <v>346</v>
       </c>
       <c r="C201" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>403</v>
+        <v>347</v>
       </c>
       <c r="B202" t="s">
-        <v>404</v>
+        <v>348</v>
       </c>
       <c r="C202" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>405</v>
+        <v>349</v>
       </c>
       <c r="B203" t="s">
-        <v>406</v>
+        <v>350</v>
       </c>
       <c r="C203" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>407</v>
+        <v>351</v>
       </c>
       <c r="B204" t="s">
-        <v>408</v>
+        <v>352</v>
       </c>
       <c r="C204" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>409</v>
+        <v>353</v>
       </c>
       <c r="B205" t="s">
-        <v>410</v>
+        <v>354</v>
       </c>
       <c r="C205" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>411</v>
+        <v>355</v>
       </c>
       <c r="B206" t="s">
-        <v>412</v>
+        <v>356</v>
       </c>
       <c r="C206" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>413</v>
+        <v>357</v>
       </c>
       <c r="B207" t="s">
-        <v>414</v>
+        <v>358</v>
       </c>
       <c r="C207" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>415</v>
+        <v>359</v>
       </c>
       <c r="B208" t="s">
-        <v>416</v>
+        <v>360</v>
       </c>
       <c r="C208" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>417</v>
+        <v>361</v>
       </c>
       <c r="B209" t="s">
-        <v>418</v>
+        <v>362</v>
       </c>
       <c r="C209" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>419</v>
+        <v>363</v>
       </c>
       <c r="B210" t="s">
-        <v>420</v>
+        <v>364</v>
       </c>
       <c r="C210" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>421</v>
+        <v>365</v>
       </c>
       <c r="B211" t="s">
-        <v>422</v>
+        <v>366</v>
       </c>
       <c r="C211" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>423</v>
+        <v>367</v>
       </c>
       <c r="B212" t="s">
-        <v>424</v>
+        <v>368</v>
       </c>
       <c r="C212" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>425</v>
+        <v>369</v>
       </c>
       <c r="B213" t="s">
-        <v>426</v>
+        <v>370</v>
       </c>
       <c r="C213" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>427</v>
+        <v>371</v>
       </c>
       <c r="B214" t="s">
-        <v>428</v>
+        <v>372</v>
       </c>
       <c r="C214" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>429</v>
+        <v>373</v>
       </c>
       <c r="B215" t="s">
-        <v>430</v>
+        <v>374</v>
       </c>
       <c r="C215" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>431</v>
+        <v>375</v>
       </c>
       <c r="B216" t="s">
-        <v>432</v>
+        <v>376</v>
       </c>
       <c r="C216" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>433</v>
+        <v>377</v>
       </c>
       <c r="B217" t="s">
-        <v>434</v>
+        <v>378</v>
       </c>
       <c r="C217" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>435</v>
+        <v>379</v>
       </c>
       <c r="B218" t="s">
-        <v>436</v>
+        <v>380</v>
       </c>
       <c r="C218" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>437</v>
+        <v>381</v>
       </c>
       <c r="B219" t="s">
-        <v>438</v>
+        <v>382</v>
       </c>
       <c r="C219" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>439</v>
+        <v>383</v>
       </c>
       <c r="B220" t="s">
-        <v>440</v>
+        <v>384</v>
       </c>
       <c r="C220" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>441</v>
+        <v>385</v>
       </c>
       <c r="B221" t="s">
-        <v>442</v>
+        <v>386</v>
       </c>
       <c r="C221" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>443</v>
+        <v>387</v>
       </c>
       <c r="B222" t="s">
-        <v>444</v>
+        <v>388</v>
       </c>
       <c r="C222" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>445</v>
+        <v>389</v>
       </c>
       <c r="B223" t="s">
-        <v>446</v>
+        <v>390</v>
       </c>
       <c r="C223" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>447</v>
+        <v>391</v>
       </c>
       <c r="B224" t="s">
-        <v>448</v>
+        <v>392</v>
       </c>
       <c r="C224" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>